<commit_message>
Verify Panatta equipment with browser evidence
- Match 164 Panatta models with official names and images
- Preserve browser evidence when HTTP requests fail
- Refresh catalog, Markdown and Excel reports
- Add regression tests for browser evidence matching
</commit_message>
<xml_diff>
--- a/docs/data/247-fitness-hk-official-equipment-research-2026-10-28.xlsx
+++ b/docs/data/247-fitness-hk-official-equipment-research-2026-10-28.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Totals" sheetId="1" r:id="R61b3f9c28f0b4794"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage by brand" sheetId="2" r:id="R0ae7804715b44f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full inventory cross-reference" sheetId="3" r:id="R15ba272e804c4b57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Totals" sheetId="1" r:id="Rcb1a24ff9eb640a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage by brand" sheetId="2" r:id="R264f688c70fc4da0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full inventory cross-reference" sheetId="3" r:id="R61cdb8e5ac124db8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -130,8 +130,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EquipmentResearch1" displayName="EquipmentResearch1" ref="A4:B9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:B9"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EquipmentResearch1" displayName="EquipmentResearch1" ref="A4:B8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:B8"/>
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Count"/>
@@ -406,7 +406,7 @@
         <x:v>candidate_requires_review</x:v>
       </x:c>
       <x:c r="B6" s="13" t="n">
-        <x:v>208</x:v>
+        <x:v>206</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
@@ -414,29 +414,21 @@
         <x:v>model_verified</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
-        <x:v>279</x:v>
+        <x:v>443</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>unresolved</x:v>
       </x:c>
       <x:c r="B8" s="13" t="n">
-        <x:v>155</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="12" t="str">
-        <x:v>unresolved</x:v>
-      </x:c>
-      <x:c r="B9" s="13" t="n">
-        <x:v>175</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re80fc1825a8e43a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb607d85d1c94288"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -988,19 +980,19 @@
         <x:v>176</x:v>
       </x:c>
       <x:c r="C26" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="D26" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E26" s="13" t="n">
-        <x:v>155</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F26" s="13" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G26" s="13" t="n">
         <x:v>7</x:v>
-      </x:c>
-      <x:c r="G26" s="13" t="n">
-        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
@@ -1328,7 +1320,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1cde9174aaf420e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ab7212a27d0452b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18650,16 +18642,16 @@
         <x:v>Total Back</x:v>
       </x:c>
       <x:c r="F497" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>Total Back</x:v>
       </x:c>
       <x:c r="G497" s="12" t="str">
-        <x:v>unresolved</x:v>
-      </x:c>
-      <x:c r="H497" s="12" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I497" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>model_verified</x:v>
+      </x:c>
+      <x:c r="H497" s="17" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="I497" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J497" s="17" t="str">
         <x:v>image</x:v>
@@ -18688,13 +18680,13 @@
         <x:v>Lat pulldown</x:v>
       </x:c>
       <x:c r="G498" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H498" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I498" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I498" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J498" s="17" t="str">
         <x:v>image</x:v>
@@ -18723,13 +18715,13 @@
         <x:v>Lat pulldown double Stack</x:v>
       </x:c>
       <x:c r="G499" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H499" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I499" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I499" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J499" s="17" t="str">
         <x:v>image</x:v>
@@ -18758,13 +18750,13 @@
         <x:v>Lat pulldown circular</x:v>
       </x:c>
       <x:c r="G500" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H500" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I500" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I500" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J500" s="17" t="str">
         <x:v>image</x:v>
@@ -18793,13 +18785,13 @@
         <x:v>Pulley row</x:v>
       </x:c>
       <x:c r="G501" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H501" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I501" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I501" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J501" s="17" t="str">
         <x:v>image</x:v>
@@ -18828,13 +18820,13 @@
         <x:v>Rowing machine circular</x:v>
       </x:c>
       <x:c r="G502" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H502" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I502" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I502" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J502" s="17" t="str">
         <x:v>image</x:v>
@@ -18863,13 +18855,13 @@
         <x:v>Deltoid press</x:v>
       </x:c>
       <x:c r="G503" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H503" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I503" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I503" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J503" s="17" t="str">
         <x:v>image</x:v>
@@ -18898,13 +18890,13 @@
         <x:v>Deltoid press circular</x:v>
       </x:c>
       <x:c r="G504" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H504" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I504" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I504" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J504" s="17" t="str">
         <x:v>image</x:v>
@@ -18933,13 +18925,13 @@
         <x:v>Vertical chest press</x:v>
       </x:c>
       <x:c r="G505" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H505" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I505" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I505" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J505" s="17" t="str">
         <x:v>image</x:v>
@@ -18968,13 +18960,13 @@
         <x:v>Inclined chest press circular</x:v>
       </x:c>
       <x:c r="G506" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H506" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I506" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I506" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J506" s="17" t="str">
         <x:v>image</x:v>
@@ -19003,13 +18995,13 @@
         <x:v>Dips press</x:v>
       </x:c>
       <x:c r="G507" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H507" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I507" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I507" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J507" s="17" t="str">
         <x:v>image</x:v>
@@ -19038,13 +19030,13 @@
         <x:v>Triceps machine</x:v>
       </x:c>
       <x:c r="G508" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H508" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I508" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I508" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J508" s="17" t="str">
         <x:v>image</x:v>
@@ -19073,13 +19065,13 @@
         <x:v>Curling machine</x:v>
       </x:c>
       <x:c r="G509" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H509" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I509" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I509" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J509" s="17" t="str">
         <x:v>image</x:v>
@@ -19108,13 +19100,13 @@
         <x:v>Alternate arm curl 120</x:v>
       </x:c>
       <x:c r="G510" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H510" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I510" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I510" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J510" s="17" t="str">
         <x:v>image</x:v>
@@ -19143,13 +19135,13 @@
         <x:v>Alternate arm curl -45</x:v>
       </x:c>
       <x:c r="G511" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H511" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I511" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I511" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J511" s="17" t="str">
         <x:v>image</x:v>
@@ -19178,13 +19170,13 @@
         <x:v>Abdominal crunch</x:v>
       </x:c>
       <x:c r="G512" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H512" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I512" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I512" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J512" s="17" t="str">
         <x:v>image</x:v>
@@ -19213,13 +19205,13 @@
         <x:v>Torsion machine</x:v>
       </x:c>
       <x:c r="G513" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H513" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I513" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I513" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J513" s="17" t="str">
         <x:v>image</x:v>
@@ -19248,13 +19240,13 @@
         <x:v>Leg extension</x:v>
       </x:c>
       <x:c r="G514" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H514" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I514" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I514" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J514" s="17" t="str">
         <x:v>image</x:v>
@@ -19283,13 +19275,13 @@
         <x:v>Leg curling</x:v>
       </x:c>
       <x:c r="G515" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H515" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I515" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I515" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J515" s="17" t="str">
         <x:v>image</x:v>
@@ -19318,13 +19310,13 @@
         <x:v>Seated leg curling</x:v>
       </x:c>
       <x:c r="G516" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H516" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I516" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I516" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J516" s="17" t="str">
         <x:v>image</x:v>
@@ -19353,13 +19345,13 @@
         <x:v>Standing leg curling</x:v>
       </x:c>
       <x:c r="G517" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H517" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I517" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I517" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J517" s="17" t="str">
         <x:v>image</x:v>
@@ -19388,13 +19380,13 @@
         <x:v>Dual system horizontal leg press</x:v>
       </x:c>
       <x:c r="G518" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H518" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I518" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I518" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J518" s="17" t="str">
         <x:v>image</x:v>
@@ -19423,13 +19415,13 @@
         <x:v>Horizontal leg press</x:v>
       </x:c>
       <x:c r="G519" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H519" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I519" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I519" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J519" s="17" t="str">
         <x:v>image</x:v>
@@ -19458,13 +19450,13 @@
         <x:v>Abductor machine</x:v>
       </x:c>
       <x:c r="G520" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H520" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I520" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I520" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J520" s="17" t="str">
         <x:v>image</x:v>
@@ -19493,13 +19485,13 @@
         <x:v>Adductor machine</x:v>
       </x:c>
       <x:c r="G521" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H521" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I521" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I521" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J521" s="17" t="str">
         <x:v>image</x:v>
@@ -19528,13 +19520,13 @@
         <x:v>Adductor/ abductor machine</x:v>
       </x:c>
       <x:c r="G522" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H522" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I522" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I522" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J522" s="17" t="str">
         <x:v>image</x:v>
@@ -19563,13 +19555,13 @@
         <x:v>Master gluteus plus</x:v>
       </x:c>
       <x:c r="G523" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H523" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I523" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I523" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J523" s="17" t="str">
         <x:v>image</x:v>
@@ -19598,13 +19590,13 @@
         <x:v>Gluteus machine</x:v>
       </x:c>
       <x:c r="G524" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H524" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I524" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I524" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J524" s="17" t="str">
         <x:v>image</x:v>
@@ -19633,13 +19625,13 @@
         <x:v>Hip thrust</x:v>
       </x:c>
       <x:c r="G525" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H525" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I525" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I525" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J525" s="17" t="str">
         <x:v>image</x:v>
@@ -19668,13 +19660,13 @@
         <x:v>Calf machine</x:v>
       </x:c>
       <x:c r="G526" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H526" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I526" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I526" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J526" s="17" t="str">
         <x:v>image</x:v>
@@ -19700,16 +19692,16 @@
         <x:v>Standing abductor machine</x:v>
       </x:c>
       <x:c r="F527" s="12" t="str">
-        <x:v>Standing abductor machine</x:v>
+        <x:v>Standing  abductor machine</x:v>
       </x:c>
       <x:c r="G527" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H527" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I527" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I527" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J527" s="17" t="str">
         <x:v>image</x:v>
@@ -19738,13 +19730,13 @@
         <x:v>Standing Total Arms</x:v>
       </x:c>
       <x:c r="G528" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H528" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I528" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I528" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J528" s="17" t="str">
         <x:v>image</x:v>
@@ -19773,13 +19765,13 @@
         <x:v>Multipurpose press</x:v>
       </x:c>
       <x:c r="G529" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H529" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I529" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I529" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J529" s="17" t="str">
         <x:v>image</x:v>
@@ -19808,13 +19800,13 @@
         <x:v>Peck back</x:v>
       </x:c>
       <x:c r="G530" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H530" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I530" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I530" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J530" s="17" t="str">
         <x:v>image</x:v>
@@ -19843,13 +19835,13 @@
         <x:v>Chin and dip counterbalanced</x:v>
       </x:c>
       <x:c r="G531" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H531" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I531" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I531" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J531" s="17" t="str">
         <x:v>image</x:v>
@@ -19878,13 +19870,13 @@
         <x:v>Flat bench</x:v>
       </x:c>
       <x:c r="G532" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H532" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I532" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I532" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J532" s="17" t="str">
         <x:v>image</x:v>
@@ -19913,13 +19905,13 @@
         <x:v>Adjustable crunch board</x:v>
       </x:c>
       <x:c r="G533" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H533" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I533" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I533" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J533" s="17" t="str">
         <x:v>image</x:v>
@@ -19948,13 +19940,13 @@
         <x:v>Iperextension 45° bench</x:v>
       </x:c>
       <x:c r="G534" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H534" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I534" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I534" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J534" s="17" t="str">
         <x:v>image</x:v>
@@ -19983,13 +19975,13 @@
         <x:v>Squat rack</x:v>
       </x:c>
       <x:c r="G535" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H535" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I535" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I535" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J535" s="17" t="str">
         <x:v>image</x:v>
@@ -20018,13 +20010,13 @@
         <x:v>Fully adjustable bench</x:v>
       </x:c>
       <x:c r="G536" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H536" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I536" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I536" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J536" s="17" t="str">
         <x:v>image</x:v>
@@ -20053,13 +20045,13 @@
         <x:v>Chin and dip</x:v>
       </x:c>
       <x:c r="G537" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H537" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I537" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I537" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J537" s="17" t="str">
         <x:v>image</x:v>
@@ -20088,13 +20080,13 @@
         <x:v>Power tower</x:v>
       </x:c>
       <x:c r="G538" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H538" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I538" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I538" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J538" s="17" t="str">
         <x:v>image</x:v>
@@ -20123,13 +20115,13 @@
         <x:v>Multipurpose seated bench</x:v>
       </x:c>
       <x:c r="G539" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H539" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I539" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I539" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J539" s="17" t="str">
         <x:v>image</x:v>
@@ -20158,13 +20150,13 @@
         <x:v>Sissy squat</x:v>
       </x:c>
       <x:c r="G540" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H540" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I540" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I540" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J540" s="17" t="str">
         <x:v>image</x:v>
@@ -20193,13 +20185,13 @@
         <x:v>Powerlifting bench</x:v>
       </x:c>
       <x:c r="G541" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H541" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I541" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I541" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J541" s="17" t="str">
         <x:v>image</x:v>
@@ -20228,13 +20220,13 @@
         <x:v>Lat pulldown circular</x:v>
       </x:c>
       <x:c r="G542" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H542" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I542" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I542" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J542" s="17" t="str">
         <x:v>image</x:v>
@@ -20263,13 +20255,13 @@
         <x:v>Lat pulldown convergent</x:v>
       </x:c>
       <x:c r="G543" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H543" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I543" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I543" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J543" s="17" t="str">
         <x:v>image</x:v>
@@ -20298,13 +20290,13 @@
         <x:v>High row convergent</x:v>
       </x:c>
       <x:c r="G544" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H544" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I544" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I544" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J544" s="17" t="str">
         <x:v>image</x:v>
@@ -20333,13 +20325,13 @@
         <x:v>Rowing machine circular</x:v>
       </x:c>
       <x:c r="G545" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H545" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I545" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I545" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J545" s="17" t="str">
         <x:v>image</x:v>
@@ -20368,13 +20360,13 @@
         <x:v>Deltoid press circular</x:v>
       </x:c>
       <x:c r="G546" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H546" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I546" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I546" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J546" s="17" t="str">
         <x:v>image</x:v>
@@ -20403,13 +20395,13 @@
         <x:v>Vertical chest press circular</x:v>
       </x:c>
       <x:c r="G547" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H547" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I547" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I547" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J547" s="17" t="str">
         <x:v>image</x:v>
@@ -20438,13 +20430,13 @@
         <x:v>Inclined chest press circular</x:v>
       </x:c>
       <x:c r="G548" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H548" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I548" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I548" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J548" s="17" t="str">
         <x:v>image</x:v>
@@ -20473,13 +20465,13 @@
         <x:v>Alternate arm extension</x:v>
       </x:c>
       <x:c r="G549" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H549" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I549" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I549" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J549" s="17" t="str">
         <x:v>image</x:v>
@@ -20508,13 +20500,13 @@
         <x:v>Abdominal crunch</x:v>
       </x:c>
       <x:c r="G550" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H550" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I550" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I550" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J550" s="17" t="str">
         <x:v>image</x:v>
@@ -20543,13 +20535,13 @@
         <x:v>Horizontal Adjustable leg press</x:v>
       </x:c>
       <x:c r="G551" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H551" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I551" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I551" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J551" s="17" t="str">
         <x:v>image</x:v>
@@ -20578,13 +20570,13 @@
         <x:v>Gluteus machine</x:v>
       </x:c>
       <x:c r="G552" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H552" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I552" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I552" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J552" s="17" t="str">
         <x:v>image</x:v>
@@ -20613,13 +20605,13 @@
         <x:v>Hip thrust</x:v>
       </x:c>
       <x:c r="G553" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H553" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I553" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I553" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J553" s="17" t="str">
         <x:v>image</x:v>
@@ -20648,13 +20640,13 @@
         <x:v>Jungle machine</x:v>
       </x:c>
       <x:c r="G554" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H554" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I554" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I554" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J554" s="17" t="str">
         <x:v>image</x:v>
@@ -20683,13 +20675,13 @@
         <x:v>Standing multi flight</x:v>
       </x:c>
       <x:c r="G555" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H555" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I555" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I555" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J555" s="17" t="str">
         <x:v>image</x:v>
@@ -20718,13 +20710,13 @@
         <x:v>Lat pulldown</x:v>
       </x:c>
       <x:c r="G556" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H556" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I556" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I556" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J556" s="17" t="str">
         <x:v>image</x:v>
@@ -20753,13 +20745,13 @@
         <x:v>Pulley row</x:v>
       </x:c>
       <x:c r="G557" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H557" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I557" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I557" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J557" s="17" t="str">
         <x:v>image</x:v>
@@ -20788,13 +20780,13 @@
         <x:v>Inclined chest press</x:v>
       </x:c>
       <x:c r="G558" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H558" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I558" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I558" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J558" s="17" t="str">
         <x:v>image</x:v>
@@ -20823,13 +20815,13 @@
         <x:v>Deltoid press convergent</x:v>
       </x:c>
       <x:c r="G559" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H559" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I559" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I559" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J559" s="17" t="str">
         <x:v>image</x:v>
@@ -20858,13 +20850,13 @@
         <x:v>Curling machine</x:v>
       </x:c>
       <x:c r="G560" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H560" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I560" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I560" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J560" s="17" t="str">
         <x:v>image</x:v>
@@ -20893,13 +20885,13 @@
         <x:v>Upper abdominal</x:v>
       </x:c>
       <x:c r="G561" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H561" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I561" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I561" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J561" s="17" t="str">
         <x:v>image</x:v>
@@ -20928,13 +20920,13 @@
         <x:v>Multi hip</x:v>
       </x:c>
       <x:c r="G562" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H562" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I562" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I562" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J562" s="17" t="str">
         <x:v>image</x:v>
@@ -20963,13 +20955,13 @@
         <x:v>Jungle machine</x:v>
       </x:c>
       <x:c r="G563" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H563" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I563" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I563" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J563" s="17" t="str">
         <x:v>image</x:v>
@@ -20998,13 +20990,13 @@
         <x:v>Chin and dip (chin optional)</x:v>
       </x:c>
       <x:c r="G564" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H564" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I564" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I564" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J564" s="17" t="str">
         <x:v>image</x:v>
@@ -21033,22 +21025,22 @@
         <x:v>Hip thrust bench</x:v>
       </x:c>
       <x:c r="G565" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H565" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I565" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I565" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J565" s="17" t="str">
         <x:v>image</x:v>
       </x:c>
-      <x:c r="K565" s="17" t="str">
-        <x:v>Hip thrust bench | Panatta Sport</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="566" ht="36" customHeight="1">
+      <x:c r="K565" s="12" t="str">
+        <x:v>—</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="566" ht="24" customHeight="1">
       <x:c r="A566" s="13" t="n">
         <x:v>562</x:v>
       </x:c>
@@ -21068,19 +21060,19 @@
         <x:v>Dual curling | triceps machine</x:v>
       </x:c>
       <x:c r="G566" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H566" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I566" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I566" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J566" s="17" t="str">
         <x:v>image</x:v>
       </x:c>
-      <x:c r="K566" s="17" t="str">
-        <x:v>Dual curling | triceps machine | Panatta Sport</x:v>
+      <x:c r="K566" s="12" t="str">
+        <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="567" ht="24" customHeight="1">
@@ -21103,19 +21095,19 @@
         <x:v>Multi press</x:v>
       </x:c>
       <x:c r="G567" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H567" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I567" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I567" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J567" s="17" t="str">
         <x:v>image</x:v>
       </x:c>
-      <x:c r="K567" s="17" t="str">
-        <x:v>Multi press | Panatta Sport</x:v>
+      <x:c r="K567" s="12" t="str">
+        <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="568" ht="24" customHeight="1">
@@ -21138,22 +21130,22 @@
         <x:v>Dual abdominal | lower back</x:v>
       </x:c>
       <x:c r="G568" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H568" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I568" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I568" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J568" s="17" t="str">
         <x:v>image</x:v>
       </x:c>
-      <x:c r="K568" s="17" t="str">
-        <x:v>Dual abdominal | lower back | Panatta Sport</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="569" ht="36" customHeight="1">
+      <x:c r="K568" s="12" t="str">
+        <x:v>—</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="569" ht="24" customHeight="1">
       <x:c r="A569" s="13" t="n">
         <x:v>565</x:v>
       </x:c>
@@ -21173,19 +21165,19 @@
         <x:v>Dual leg extension | seated leg curling</x:v>
       </x:c>
       <x:c r="G569" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H569" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I569" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I569" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J569" s="17" t="str">
         <x:v>image</x:v>
       </x:c>
-      <x:c r="K569" s="17" t="str">
-        <x:v>Dual leg extension | seated leg curling | Panatta Sport</x:v>
+      <x:c r="K569" s="12" t="str">
+        <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="570" ht="24" customHeight="1">
@@ -21205,16 +21197,16 @@
         <x:v>DIPS PRESS</x:v>
       </x:c>
       <x:c r="F570" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>Dips Press</x:v>
       </x:c>
       <x:c r="G570" s="12" t="str">
-        <x:v>unresolved</x:v>
-      </x:c>
-      <x:c r="H570" s="12" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I570" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>model_verified</x:v>
+      </x:c>
+      <x:c r="H570" s="17" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="I570" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J570" s="17" t="str">
         <x:v>image</x:v>
@@ -21240,16 +21232,16 @@
         <x:v>POWER SMITH MACHINE  MULTI ANGLES</x:v>
       </x:c>
       <x:c r="F571" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>Power Smith Machine Multi Angles</x:v>
       </x:c>
       <x:c r="G571" s="12" t="str">
-        <x:v>unresolved</x:v>
-      </x:c>
-      <x:c r="H571" s="12" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I571" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>model_verified</x:v>
+      </x:c>
+      <x:c r="H571" s="17" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="I571" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J571" s="17" t="str">
         <x:v>image</x:v>
@@ -21275,16 +21267,16 @@
         <x:v>SQUAT MACHINE AND CALF</x:v>
       </x:c>
       <x:c r="F572" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>Squat and Calf Machine</x:v>
       </x:c>
       <x:c r="G572" s="12" t="str">
-        <x:v>unresolved</x:v>
-      </x:c>
-      <x:c r="H572" s="12" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I572" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>model_verified</x:v>
+      </x:c>
+      <x:c r="H572" s="17" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="I572" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J572" s="17" t="str">
         <x:v>image</x:v>
@@ -21310,16 +21302,16 @@
         <x:v>HACK SQUAT</x:v>
       </x:c>
       <x:c r="F573" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>Hack Squat</x:v>
       </x:c>
       <x:c r="G573" s="12" t="str">
-        <x:v>unresolved</x:v>
-      </x:c>
-      <x:c r="H573" s="12" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I573" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>model_verified</x:v>
+      </x:c>
+      <x:c r="H573" s="17" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="I573" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J573" s="17" t="str">
         <x:v>image</x:v>
@@ -21348,13 +21340,13 @@
         <x:v>Kneeling leg curling</x:v>
       </x:c>
       <x:c r="G574" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H574" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I574" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I574" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J574" s="17" t="str">
         <x:v>image</x:v>
@@ -21383,13 +21375,13 @@
         <x:v>Middle chest flight machine</x:v>
       </x:c>
       <x:c r="G575" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H575" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I575" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I575" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J575" s="17" t="str">
         <x:v>image</x:v>
@@ -21418,13 +21410,13 @@
         <x:v>Pullover machine</x:v>
       </x:c>
       <x:c r="G576" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H576" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I576" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I576" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J576" s="17" t="str">
         <x:v>image</x:v>
@@ -21453,13 +21445,13 @@
         <x:v>Lat pulldown circular</x:v>
       </x:c>
       <x:c r="G577" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H577" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I577" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I577" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J577" s="17" t="str">
         <x:v>image</x:v>
@@ -21488,13 +21480,13 @@
         <x:v>Hip thrust</x:v>
       </x:c>
       <x:c r="G578" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H578" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I578" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I578" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J578" s="17" t="str">
         <x:v>image</x:v>
@@ -21523,13 +21515,13 @@
         <x:v>Leg press bridge</x:v>
       </x:c>
       <x:c r="G579" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H579" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I579" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I579" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J579" s="17" t="str">
         <x:v>image</x:v>
@@ -21558,13 +21550,13 @@
         <x:v>Upper Chest Flight Machine</x:v>
       </x:c>
       <x:c r="G580" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H580" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I580" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I580" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J580" s="17" t="str">
         <x:v>image</x:v>
@@ -21593,13 +21585,13 @@
         <x:v>Lat machine convergent</x:v>
       </x:c>
       <x:c r="G581" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H581" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I581" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I581" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J581" s="17" t="str">
         <x:v>image</x:v>
@@ -21628,13 +21620,13 @@
         <x:v>Rowing machine</x:v>
       </x:c>
       <x:c r="G582" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H582" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I582" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I582" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J582" s="17" t="str">
         <x:v>image</x:v>
@@ -21663,13 +21655,13 @@
         <x:v>Low row</x:v>
       </x:c>
       <x:c r="G583" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H583" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I583" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I583" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J583" s="17" t="str">
         <x:v>image</x:v>
@@ -21698,13 +21690,13 @@
         <x:v>High row</x:v>
       </x:c>
       <x:c r="G584" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H584" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I584" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I584" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J584" s="17" t="str">
         <x:v>image</x:v>
@@ -21733,13 +21725,13 @@
         <x:v>Deltoid press</x:v>
       </x:c>
       <x:c r="G585" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H585" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I585" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I585" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J585" s="17" t="str">
         <x:v>image</x:v>
@@ -21768,13 +21760,13 @@
         <x:v>Leg press 45°</x:v>
       </x:c>
       <x:c r="G586" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H586" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I586" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I586" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J586" s="17" t="str">
         <x:v>image</x:v>
@@ -21803,13 +21795,13 @@
         <x:v>Pendulum squat</x:v>
       </x:c>
       <x:c r="G587" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H587" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I587" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I587" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J587" s="17" t="str">
         <x:v>image</x:v>
@@ -21873,13 +21865,13 @@
         <x:v>Three Angles Triceps Machine</x:v>
       </x:c>
       <x:c r="G589" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H589" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I589" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I589" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J589" s="17" t="str">
         <x:v>image</x:v>
@@ -21908,13 +21900,13 @@
         <x:v>Alternate Arm Curl 120</x:v>
       </x:c>
       <x:c r="G590" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H590" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I590" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I590" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J590" s="17" t="str">
         <x:v>image</x:v>
@@ -21940,16 +21932,16 @@
         <x:v>3D ABDUCTOR</x:v>
       </x:c>
       <x:c r="F591" s="12" t="str">
-        <x:v>3D ABDUCTOR</x:v>
+        <x:v>3D Abductor</x:v>
       </x:c>
       <x:c r="G591" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H591" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I591" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I591" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J591" s="17" t="str">
         <x:v>image</x:v>
@@ -21975,16 +21967,16 @@
         <x:v>POWER SMITH DUAL SYSTEM UPPER</x:v>
       </x:c>
       <x:c r="F592" s="12" t="str">
-        <x:v>POWER SMITH MACHINE DUAL SYSTEM UPPER</x:v>
+        <x:v>Power smith dual system upper</x:v>
       </x:c>
       <x:c r="G592" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H592" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I592" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I592" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J592" s="17" t="str">
         <x:v>image</x:v>
@@ -22010,16 +22002,16 @@
         <x:v>TOTAL CORE CRUNCH MACHINE</x:v>
       </x:c>
       <x:c r="F593" s="12" t="str">
-        <x:v>TOTAL CORE CRUNCH MACHINE</x:v>
+        <x:v>Total core crunch machine</x:v>
       </x:c>
       <x:c r="G593" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H593" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I593" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I593" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J593" s="17" t="str">
         <x:v>image</x:v>
@@ -22045,16 +22037,16 @@
         <x:v>SUPER VERTICAL MULTI PRESS</x:v>
       </x:c>
       <x:c r="F594" s="12" t="str">
-        <x:v>SUPER VERTICAL MULTI PRESS</x:v>
+        <x:v>Super vertical multi press</x:v>
       </x:c>
       <x:c r="G594" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H594" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I594" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I594" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J594" s="17" t="str">
         <x:v>image</x:v>
@@ -22083,13 +22075,13 @@
         <x:v>Super vertical chest press</x:v>
       </x:c>
       <x:c r="G595" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H595" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I595" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I595" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J595" s="17" t="str">
         <x:v>image</x:v>
@@ -22118,13 +22110,13 @@
         <x:v>Super inclined chest press</x:v>
       </x:c>
       <x:c r="G596" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H596" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I596" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I596" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J596" s="17" t="str">
         <x:v>image</x:v>
@@ -22153,13 +22145,13 @@
         <x:v>Super declined chest press</x:v>
       </x:c>
       <x:c r="G597" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H597" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I597" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I597" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J597" s="17" t="str">
         <x:v>image</x:v>
@@ -22188,19 +22180,19 @@
         <x:v>Super Horizontal Bench Press</x:v>
       </x:c>
       <x:c r="G598" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H598" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I598" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I598" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J598" s="17" t="str">
         <x:v>image</x:v>
       </x:c>
-      <x:c r="K598" s="17" t="str">
-        <x:v>Super Horizontal Bench Press | Panatta Sport</x:v>
+      <x:c r="K598" s="12" t="str">
+        <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="599" ht="24" customHeight="1">
@@ -22223,13 +22215,13 @@
         <x:v>Super inclined bench press</x:v>
       </x:c>
       <x:c r="G599" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H599" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I599" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I599" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J599" s="17" t="str">
         <x:v>image</x:v>
@@ -22258,13 +22250,13 @@
         <x:v>Super middle chest flight machine</x:v>
       </x:c>
       <x:c r="G600" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H600" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I600" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I600" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J600" s="17" t="str">
         <x:v>image</x:v>
@@ -22293,13 +22285,13 @@
         <x:v>Super upper chest flight machine</x:v>
       </x:c>
       <x:c r="G601" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H601" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I601" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I601" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J601" s="17" t="str">
         <x:v>image</x:v>
@@ -22328,13 +22320,13 @@
         <x:v>Super lower chest flight machine</x:v>
       </x:c>
       <x:c r="G602" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H602" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I602" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I602" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J602" s="17" t="str">
         <x:v>image</x:v>
@@ -22363,13 +22355,13 @@
         <x:v>Super horizontal multi press</x:v>
       </x:c>
       <x:c r="G603" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H603" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I603" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I603" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J603" s="17" t="str">
         <x:v>image</x:v>
@@ -22398,13 +22390,13 @@
         <x:v>Dips press dual system</x:v>
       </x:c>
       <x:c r="G604" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H604" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I604" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I604" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J604" s="17" t="str">
         <x:v>image</x:v>
@@ -22433,13 +22425,13 @@
         <x:v>Dips press</x:v>
       </x:c>
       <x:c r="G605" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H605" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I605" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I605" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J605" s="17" t="str">
         <x:v>image</x:v>
@@ -22468,13 +22460,13 @@
         <x:v>Super pullover machine</x:v>
       </x:c>
       <x:c r="G606" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H606" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I606" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I606" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J606" s="17" t="str">
         <x:v>image</x:v>
@@ -22503,13 +22495,13 @@
         <x:v>Pullover machine</x:v>
       </x:c>
       <x:c r="G607" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H607" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I607" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I607" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J607" s="17" t="str">
         <x:v>image</x:v>
@@ -22538,13 +22530,13 @@
         <x:v>Super lat machine convergent</x:v>
       </x:c>
       <x:c r="G608" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H608" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I608" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I608" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J608" s="17" t="str">
         <x:v>image</x:v>
@@ -22573,13 +22565,13 @@
         <x:v>Super lat pulldown circular</x:v>
       </x:c>
       <x:c r="G609" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H609" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I609" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I609" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J609" s="17" t="str">
         <x:v>image</x:v>
@@ -22608,13 +22600,13 @@
         <x:v>Super high row</x:v>
       </x:c>
       <x:c r="G610" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H610" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I610" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I610" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J610" s="17" t="str">
         <x:v>image</x:v>
@@ -22643,13 +22635,13 @@
         <x:v>Super power row</x:v>
       </x:c>
       <x:c r="G611" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H611" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I611" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I611" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J611" s="17" t="str">
         <x:v>image</x:v>
@@ -22678,13 +22670,13 @@
         <x:v>Super low row</x:v>
       </x:c>
       <x:c r="G612" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H612" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I612" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I612" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J612" s="17" t="str">
         <x:v>image</x:v>
@@ -22713,13 +22705,13 @@
         <x:v>Super Rowing</x:v>
       </x:c>
       <x:c r="G613" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H613" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I613" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I613" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J613" s="17" t="str">
         <x:v>image</x:v>
@@ -22745,16 +22737,16 @@
         <x:v>SUPER ROWING CIRCULAR</x:v>
       </x:c>
       <x:c r="F614" s="12" t="str">
-        <x:v>SUPER ROWING MACHINE CIRCULAR</x:v>
+        <x:v>Super rowing circular</x:v>
       </x:c>
       <x:c r="G614" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H614" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I614" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I614" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J614" s="17" t="str">
         <x:v>image</x:v>
@@ -22783,13 +22775,13 @@
         <x:v>T-bar row</x:v>
       </x:c>
       <x:c r="G615" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H615" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I615" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I615" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J615" s="17" t="str">
         <x:v>image</x:v>
@@ -22818,13 +22810,13 @@
         <x:v>Front dorsy bar</x:v>
       </x:c>
       <x:c r="G616" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H616" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I616" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I616" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J616" s="17" t="str">
         <x:v>image</x:v>
@@ -22853,13 +22845,13 @@
         <x:v>Super deltoid press</x:v>
       </x:c>
       <x:c r="G617" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H617" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I617" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I617" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J617" s="17" t="str">
         <x:v>image</x:v>
@@ -22888,13 +22880,13 @@
         <x:v>Lateral deltoids</x:v>
       </x:c>
       <x:c r="G618" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H618" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I618" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I618" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J618" s="17" t="str">
         <x:v>image</x:v>
@@ -22923,13 +22915,13 @@
         <x:v>Back deltoids</x:v>
       </x:c>
       <x:c r="G619" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H619" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I619" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I619" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J619" s="17" t="str">
         <x:v>image</x:v>
@@ -22955,16 +22947,16 @@
         <x:v>ALTERNATE CURLING MACHINE</x:v>
       </x:c>
       <x:c r="F620" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>Alternate curling machine</x:v>
       </x:c>
       <x:c r="G620" s="12" t="str">
-        <x:v>unresolved</x:v>
-      </x:c>
-      <x:c r="H620" s="12" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I620" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>model_verified</x:v>
+      </x:c>
+      <x:c r="H620" s="17" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="I620" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J620" s="17" t="str">
         <x:v>image</x:v>
@@ -22973,7 +22965,7 @@
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="621" ht="36" customHeight="1">
+    <x:row r="621" ht="24" customHeight="1">
       <x:c r="A621" s="13" t="n">
         <x:v>617</x:v>
       </x:c>
@@ -22990,22 +22982,22 @@
         <x:v>THREE ANGLES BICEPS MACHINE</x:v>
       </x:c>
       <x:c r="F621" s="12" t="str">
-        <x:v>THREE ANGLES BICEPS MACHINE</x:v>
+        <x:v>Three Angles Biceps Machine</x:v>
       </x:c>
       <x:c r="G621" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H621" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I621" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I621" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J621" s="17" t="str">
         <x:v>image</x:v>
       </x:c>
-      <x:c r="K621" s="17" t="str">
-        <x:v>Three Angles Biceps Machine | Biceps brachii | Panatta</x:v>
+      <x:c r="K621" s="12" t="str">
+        <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="622" ht="24" customHeight="1">
@@ -23028,13 +23020,13 @@
         <x:v>Super leg press bridge</x:v>
       </x:c>
       <x:c r="G622" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H622" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I622" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I622" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J622" s="17" t="str">
         <x:v>image</x:v>
@@ -23060,16 +23052,16 @@
         <x:v>SUPER HORIZONTAL LEG PRESS  DUAL SYSTEM</x:v>
       </x:c>
       <x:c r="F623" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>Super Horizontal Leg Press Dual System</x:v>
       </x:c>
       <x:c r="G623" s="12" t="str">
-        <x:v>unresolved</x:v>
-      </x:c>
-      <x:c r="H623" s="12" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I623" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>model_verified</x:v>
+      </x:c>
+      <x:c r="H623" s="17" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="I623" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J623" s="17" t="str">
         <x:v>image</x:v>
@@ -23098,13 +23090,13 @@
         <x:v>Super leg press 45°</x:v>
       </x:c>
       <x:c r="G624" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H624" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I624" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I624" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J624" s="17" t="str">
         <x:v>image</x:v>
@@ -23133,13 +23125,13 @@
         <x:v>Super leg press 45° dual system</x:v>
       </x:c>
       <x:c r="G625" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H625" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I625" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I625" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J625" s="17" t="str">
         <x:v>image</x:v>
@@ -23168,13 +23160,13 @@
         <x:v>Super vertical leg press</x:v>
       </x:c>
       <x:c r="G626" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H626" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I626" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I626" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J626" s="17" t="str">
         <x:v>image</x:v>
@@ -23183,7 +23175,7 @@
         <x:v>—</x:v>
       </x:c>
     </x:row>
-    <x:row r="627" ht="36" customHeight="1">
+    <x:row r="627" ht="24" customHeight="1">
       <x:c r="A627" s="13" t="n">
         <x:v>623</x:v>
       </x:c>
@@ -23200,22 +23192,22 @@
         <x:v>VERTICAL LEG PRESS</x:v>
       </x:c>
       <x:c r="F627" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>Vertical leg press</x:v>
       </x:c>
       <x:c r="G627" s="12" t="str">
-        <x:v>candidate_requires_review</x:v>
-      </x:c>
-      <x:c r="H627" s="12" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I627" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>model_verified</x:v>
+      </x:c>
+      <x:c r="H627" s="17" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="I627" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J627" s="17" t="str">
         <x:v>image</x:v>
       </x:c>
-      <x:c r="K627" s="17" t="str">
-        <x:v>Vertical Leg Press | Quadriceps femorals glutes | Panatta</x:v>
+      <x:c r="K627" s="12" t="str">
+        <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="628" ht="24" customHeight="1">
@@ -23238,13 +23230,13 @@
         <x:v>Super squat machine</x:v>
       </x:c>
       <x:c r="G628" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H628" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I628" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I628" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J628" s="17" t="str">
         <x:v>image</x:v>
@@ -23273,13 +23265,13 @@
         <x:v>Super power squat</x:v>
       </x:c>
       <x:c r="G629" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H629" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I629" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I629" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J629" s="17" t="str">
         <x:v>image</x:v>
@@ -23308,13 +23300,13 @@
         <x:v>Super pendulum squat</x:v>
       </x:c>
       <x:c r="G630" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H630" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I630" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I630" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J630" s="17" t="str">
         <x:v>image</x:v>
@@ -23343,13 +23335,13 @@
         <x:v>Belt squat</x:v>
       </x:c>
       <x:c r="G631" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H631" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I631" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I631" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J631" s="17" t="str">
         <x:v>image</x:v>
@@ -23378,13 +23370,13 @@
         <x:v>Super hack squat</x:v>
       </x:c>
       <x:c r="G632" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H632" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I632" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I632" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J632" s="17" t="str">
         <x:v>image</x:v>
@@ -23413,13 +23405,13 @@
         <x:v>Power runner</x:v>
       </x:c>
       <x:c r="G633" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H633" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I633" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I633" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J633" s="17" t="str">
         <x:v>image</x:v>
@@ -23448,13 +23440,13 @@
         <x:v>Hip thrust</x:v>
       </x:c>
       <x:c r="G634" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H634" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I634" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I634" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J634" s="17" t="str">
         <x:v>image</x:v>
@@ -23483,13 +23475,13 @@
         <x:v>Standing abductor</x:v>
       </x:c>
       <x:c r="G635" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H635" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I635" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I635" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J635" s="17" t="str">
         <x:v>image</x:v>
@@ -23518,13 +23510,13 @@
         <x:v>Leg extension</x:v>
       </x:c>
       <x:c r="G636" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H636" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I636" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I636" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J636" s="17" t="str">
         <x:v>image</x:v>
@@ -23553,13 +23545,13 @@
         <x:v>Alternate leg curling</x:v>
       </x:c>
       <x:c r="G637" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H637" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I637" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I637" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J637" s="17" t="str">
         <x:v>image</x:v>
@@ -23588,13 +23580,13 @@
         <x:v>Leg curling</x:v>
       </x:c>
       <x:c r="G638" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H638" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I638" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I638" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J638" s="17" t="str">
         <x:v>image</x:v>
@@ -23623,13 +23615,13 @@
         <x:v>Kneeling leg curling</x:v>
       </x:c>
       <x:c r="G639" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H639" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I639" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I639" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J639" s="17" t="str">
         <x:v>image</x:v>
@@ -23658,13 +23650,13 @@
         <x:v>Reverse hyperextension</x:v>
       </x:c>
       <x:c r="G640" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H640" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I640" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I640" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J640" s="17" t="str">
         <x:v>image</x:v>
@@ -23690,16 +23682,16 @@
         <x:v>SUPER PECK BACK</x:v>
       </x:c>
       <x:c r="F641" s="12" t="str">
-        <x:v>SUPER PECK BACK</x:v>
+        <x:v>Super Peck Back</x:v>
       </x:c>
       <x:c r="G641" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H641" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I641" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I641" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J641" s="17" t="str">
         <x:v>image</x:v>
@@ -23728,13 +23720,13 @@
         <x:v>Viking press and calf</x:v>
       </x:c>
       <x:c r="G642" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H642" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I642" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I642" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J642" s="17" t="str">
         <x:v>image</x:v>
@@ -23763,13 +23755,13 @@
         <x:v>Olympic smith machine counterbalanced</x:v>
       </x:c>
       <x:c r="G643" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H643" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I643" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I643" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J643" s="17" t="str">
         <x:v>image</x:v>
@@ -23795,22 +23787,22 @@
         <x:v>SEAL ROW BENCH</x:v>
       </x:c>
       <x:c r="F644" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>Seal row bench</x:v>
       </x:c>
       <x:c r="G644" s="12" t="str">
-        <x:v>candidate_requires_review</x:v>
-      </x:c>
-      <x:c r="H644" s="12" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I644" s="12" t="str">
-        <x:v>—</x:v>
+        <x:v>model_verified</x:v>
+      </x:c>
+      <x:c r="H644" s="17" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="I644" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J644" s="17" t="str">
         <x:v>image</x:v>
       </x:c>
-      <x:c r="K644" s="17" t="str">
-        <x:v>Seal Row Bench | Espalda central | Panatta</x:v>
+      <x:c r="K644" s="12" t="str">
+        <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="645" ht="24" customHeight="1">
@@ -23833,13 +23825,13 @@
         <x:v>Alternate triceps machine</x:v>
       </x:c>
       <x:c r="G645" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H645" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I645" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I645" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J645" s="17" t="str">
         <x:v>image</x:v>
@@ -23903,13 +23895,13 @@
         <x:v>Standing multi flight</x:v>
       </x:c>
       <x:c r="G647" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H647" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I647" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I647" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J647" s="17" t="str">
         <x:v>image</x:v>
@@ -24043,13 +24035,13 @@
         <x:v>Dual adjustable pulley full</x:v>
       </x:c>
       <x:c r="G651" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H651" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I651" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I651" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J651" s="17" t="str">
         <x:v>image</x:v>
@@ -24078,13 +24070,13 @@
         <x:v>Ecorow</x:v>
       </x:c>
       <x:c r="G652" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H652" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I652" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I652" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J652" s="17" t="str">
         <x:v>image</x:v>
@@ -24113,13 +24105,13 @@
         <x:v>Elliptical fenix touch</x:v>
       </x:c>
       <x:c r="G653" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H653" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I653" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I653" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J653" s="17" t="str">
         <x:v>image</x:v>
@@ -24148,13 +24140,13 @@
         <x:v>Climber fenix touch</x:v>
       </x:c>
       <x:c r="G654" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H654" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I654" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I654" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J654" s="17" t="str">
         <x:v>image</x:v>
@@ -24183,13 +24175,13 @@
         <x:v>Disk Rack – Fit Evo</x:v>
       </x:c>
       <x:c r="G655" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H655" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I655" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I655" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J655" s="17" t="str">
         <x:v>image</x:v>
@@ -24218,13 +24210,13 @@
         <x:v>Barbell rack double sided</x:v>
       </x:c>
       <x:c r="G656" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H656" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I656" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I656" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J656" s="17" t="str">
         <x:v>image</x:v>
@@ -24253,19 +24245,19 @@
         <x:v>Stretching extensor bench</x:v>
       </x:c>
       <x:c r="G657" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H657" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I657" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I657" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J657" s="17" t="str">
         <x:v>image</x:v>
       </x:c>
-      <x:c r="K657" s="17" t="str">
-        <x:v>Stretching extensor bench | Panatta Sport</x:v>
+      <x:c r="K657" s="12" t="str">
+        <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="658" ht="24" customHeight="1">
@@ -24288,13 +24280,13 @@
         <x:v>Adjustable standing curl bench</x:v>
       </x:c>
       <x:c r="G658" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H658" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I658" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I658" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J658" s="17" t="str">
         <x:v>image</x:v>
@@ -24358,13 +24350,13 @@
         <x:v>Squat lunge</x:v>
       </x:c>
       <x:c r="G660" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H660" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I660" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I660" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J660" s="17" t="str">
         <x:v>image</x:v>
@@ -24393,13 +24385,13 @@
         <x:v>Olympic platform – half rack (3x3m)</x:v>
       </x:c>
       <x:c r="G661" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H661" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I661" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I661" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J661" s="17" t="str">
         <x:v>image</x:v>
@@ -24428,13 +24420,13 @@
         <x:v>Rossopuro Bike Touch</x:v>
       </x:c>
       <x:c r="G662" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H662" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I662" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I662" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J662" s="17" t="str">
         <x:v>image</x:v>
@@ -24463,13 +24455,13 @@
         <x:v>Rossopuro Horizontal Bike Touch</x:v>
       </x:c>
       <x:c r="G663" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H663" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I663" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I663" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J663" s="17" t="str">
         <x:v>image</x:v>
@@ -24498,13 +24490,13 @@
         <x:v>Rossopuro Run Touch</x:v>
       </x:c>
       <x:c r="G664" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H664" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I664" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I664" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J664" s="17" t="str">
         <x:v>image</x:v>
@@ -24533,13 +24525,13 @@
         <x:v>Jungle machine hlp</x:v>
       </x:c>
       <x:c r="G665" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H665" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I665" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I665" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J665" s="17" t="str">
         <x:v>image</x:v>
@@ -24743,13 +24735,13 @@
         <x:v>Pullover machine</x:v>
       </x:c>
       <x:c r="G671" s="12" t="str">
-        <x:v>name_indexed_image_missing</x:v>
+        <x:v>model_verified</x:v>
       </x:c>
       <x:c r="H671" s="17" t="str">
         <x:v>source</x:v>
       </x:c>
-      <x:c r="I671" s="12" t="str">
-        <x:v>—</x:v>
+      <x:c r="I671" s="17" t="str">
+        <x:v>image</x:v>
       </x:c>
       <x:c r="J671" s="17" t="str">
         <x:v>image</x:v>
@@ -31699,659 +31691,822 @@
     <x:hyperlink ref="H496" r:id="GymoryHyperlink1127"/>
     <x:hyperlink ref="I496" r:id="GymoryHyperlink1128"/>
     <x:hyperlink ref="J496" r:id="GymoryHyperlink1129"/>
-    <x:hyperlink ref="J497" r:id="GymoryHyperlink1130"/>
-    <x:hyperlink ref="H498" r:id="GymoryHyperlink1131"/>
-    <x:hyperlink ref="J498" r:id="GymoryHyperlink1132"/>
-    <x:hyperlink ref="H499" r:id="GymoryHyperlink1133"/>
-    <x:hyperlink ref="J499" r:id="GymoryHyperlink1134"/>
-    <x:hyperlink ref="H500" r:id="GymoryHyperlink1135"/>
-    <x:hyperlink ref="J500" r:id="GymoryHyperlink1136"/>
-    <x:hyperlink ref="H501" r:id="GymoryHyperlink1137"/>
-    <x:hyperlink ref="J501" r:id="GymoryHyperlink1138"/>
-    <x:hyperlink ref="H502" r:id="GymoryHyperlink1139"/>
-    <x:hyperlink ref="J502" r:id="GymoryHyperlink1140"/>
-    <x:hyperlink ref="H503" r:id="GymoryHyperlink1141"/>
-    <x:hyperlink ref="J503" r:id="GymoryHyperlink1142"/>
-    <x:hyperlink ref="H504" r:id="GymoryHyperlink1143"/>
-    <x:hyperlink ref="J504" r:id="GymoryHyperlink1144"/>
-    <x:hyperlink ref="H505" r:id="GymoryHyperlink1145"/>
-    <x:hyperlink ref="J505" r:id="GymoryHyperlink1146"/>
-    <x:hyperlink ref="H506" r:id="GymoryHyperlink1147"/>
-    <x:hyperlink ref="J506" r:id="GymoryHyperlink1148"/>
-    <x:hyperlink ref="H507" r:id="GymoryHyperlink1149"/>
-    <x:hyperlink ref="J507" r:id="GymoryHyperlink1150"/>
-    <x:hyperlink ref="H508" r:id="GymoryHyperlink1151"/>
-    <x:hyperlink ref="J508" r:id="GymoryHyperlink1152"/>
-    <x:hyperlink ref="H509" r:id="GymoryHyperlink1153"/>
-    <x:hyperlink ref="J509" r:id="GymoryHyperlink1154"/>
-    <x:hyperlink ref="H510" r:id="GymoryHyperlink1155"/>
-    <x:hyperlink ref="J510" r:id="GymoryHyperlink1156"/>
-    <x:hyperlink ref="H511" r:id="GymoryHyperlink1157"/>
-    <x:hyperlink ref="J511" r:id="GymoryHyperlink1158"/>
-    <x:hyperlink ref="H512" r:id="GymoryHyperlink1159"/>
-    <x:hyperlink ref="J512" r:id="GymoryHyperlink1160"/>
-    <x:hyperlink ref="H513" r:id="GymoryHyperlink1161"/>
-    <x:hyperlink ref="J513" r:id="GymoryHyperlink1162"/>
-    <x:hyperlink ref="H514" r:id="GymoryHyperlink1163"/>
-    <x:hyperlink ref="J514" r:id="GymoryHyperlink1164"/>
-    <x:hyperlink ref="H515" r:id="GymoryHyperlink1165"/>
-    <x:hyperlink ref="J515" r:id="GymoryHyperlink1166"/>
-    <x:hyperlink ref="H516" r:id="GymoryHyperlink1167"/>
-    <x:hyperlink ref="J516" r:id="GymoryHyperlink1168"/>
-    <x:hyperlink ref="H517" r:id="GymoryHyperlink1169"/>
-    <x:hyperlink ref="J517" r:id="GymoryHyperlink1170"/>
-    <x:hyperlink ref="H518" r:id="GymoryHyperlink1171"/>
-    <x:hyperlink ref="J518" r:id="GymoryHyperlink1172"/>
-    <x:hyperlink ref="H519" r:id="GymoryHyperlink1173"/>
-    <x:hyperlink ref="J519" r:id="GymoryHyperlink1174"/>
-    <x:hyperlink ref="H520" r:id="GymoryHyperlink1175"/>
-    <x:hyperlink ref="J520" r:id="GymoryHyperlink1176"/>
-    <x:hyperlink ref="H521" r:id="GymoryHyperlink1177"/>
-    <x:hyperlink ref="J521" r:id="GymoryHyperlink1178"/>
-    <x:hyperlink ref="H522" r:id="GymoryHyperlink1179"/>
-    <x:hyperlink ref="J522" r:id="GymoryHyperlink1180"/>
-    <x:hyperlink ref="H523" r:id="GymoryHyperlink1181"/>
-    <x:hyperlink ref="J523" r:id="GymoryHyperlink1182"/>
-    <x:hyperlink ref="H524" r:id="GymoryHyperlink1183"/>
-    <x:hyperlink ref="J524" r:id="GymoryHyperlink1184"/>
-    <x:hyperlink ref="H525" r:id="GymoryHyperlink1185"/>
-    <x:hyperlink ref="J525" r:id="GymoryHyperlink1186"/>
-    <x:hyperlink ref="H526" r:id="GymoryHyperlink1187"/>
-    <x:hyperlink ref="J526" r:id="GymoryHyperlink1188"/>
-    <x:hyperlink ref="H527" r:id="GymoryHyperlink1189"/>
-    <x:hyperlink ref="J527" r:id="GymoryHyperlink1190"/>
-    <x:hyperlink ref="H528" r:id="GymoryHyperlink1191"/>
-    <x:hyperlink ref="J528" r:id="GymoryHyperlink1192"/>
-    <x:hyperlink ref="H529" r:id="GymoryHyperlink1193"/>
-    <x:hyperlink ref="J529" r:id="GymoryHyperlink1194"/>
-    <x:hyperlink ref="H530" r:id="GymoryHyperlink1195"/>
-    <x:hyperlink ref="J530" r:id="GymoryHyperlink1196"/>
-    <x:hyperlink ref="H531" r:id="GymoryHyperlink1197"/>
-    <x:hyperlink ref="J531" r:id="GymoryHyperlink1198"/>
-    <x:hyperlink ref="H532" r:id="GymoryHyperlink1199"/>
-    <x:hyperlink ref="J532" r:id="GymoryHyperlink1200"/>
-    <x:hyperlink ref="H533" r:id="GymoryHyperlink1201"/>
-    <x:hyperlink ref="J533" r:id="GymoryHyperlink1202"/>
-    <x:hyperlink ref="H534" r:id="GymoryHyperlink1203"/>
-    <x:hyperlink ref="J534" r:id="GymoryHyperlink1204"/>
-    <x:hyperlink ref="H535" r:id="GymoryHyperlink1205"/>
-    <x:hyperlink ref="J535" r:id="GymoryHyperlink1206"/>
-    <x:hyperlink ref="H536" r:id="GymoryHyperlink1207"/>
-    <x:hyperlink ref="J536" r:id="GymoryHyperlink1208"/>
-    <x:hyperlink ref="H537" r:id="GymoryHyperlink1209"/>
-    <x:hyperlink ref="J537" r:id="GymoryHyperlink1210"/>
-    <x:hyperlink ref="H538" r:id="GymoryHyperlink1211"/>
-    <x:hyperlink ref="J538" r:id="GymoryHyperlink1212"/>
-    <x:hyperlink ref="H539" r:id="GymoryHyperlink1213"/>
-    <x:hyperlink ref="J539" r:id="GymoryHyperlink1214"/>
-    <x:hyperlink ref="H540" r:id="GymoryHyperlink1215"/>
-    <x:hyperlink ref="J540" r:id="GymoryHyperlink1216"/>
-    <x:hyperlink ref="H541" r:id="GymoryHyperlink1217"/>
-    <x:hyperlink ref="J541" r:id="GymoryHyperlink1218"/>
-    <x:hyperlink ref="H542" r:id="GymoryHyperlink1219"/>
-    <x:hyperlink ref="J542" r:id="GymoryHyperlink1220"/>
-    <x:hyperlink ref="H543" r:id="GymoryHyperlink1221"/>
-    <x:hyperlink ref="J543" r:id="GymoryHyperlink1222"/>
-    <x:hyperlink ref="H544" r:id="GymoryHyperlink1223"/>
-    <x:hyperlink ref="J544" r:id="GymoryHyperlink1224"/>
-    <x:hyperlink ref="H545" r:id="GymoryHyperlink1225"/>
-    <x:hyperlink ref="J545" r:id="GymoryHyperlink1226"/>
-    <x:hyperlink ref="H546" r:id="GymoryHyperlink1227"/>
-    <x:hyperlink ref="J546" r:id="GymoryHyperlink1228"/>
-    <x:hyperlink ref="H547" r:id="GymoryHyperlink1229"/>
-    <x:hyperlink ref="J547" r:id="GymoryHyperlink1230"/>
-    <x:hyperlink ref="H548" r:id="GymoryHyperlink1231"/>
-    <x:hyperlink ref="J548" r:id="GymoryHyperlink1232"/>
-    <x:hyperlink ref="H549" r:id="GymoryHyperlink1233"/>
-    <x:hyperlink ref="J549" r:id="GymoryHyperlink1234"/>
-    <x:hyperlink ref="H550" r:id="GymoryHyperlink1235"/>
-    <x:hyperlink ref="J550" r:id="GymoryHyperlink1236"/>
-    <x:hyperlink ref="H551" r:id="GymoryHyperlink1237"/>
-    <x:hyperlink ref="J551" r:id="GymoryHyperlink1238"/>
-    <x:hyperlink ref="H552" r:id="GymoryHyperlink1239"/>
-    <x:hyperlink ref="J552" r:id="GymoryHyperlink1240"/>
-    <x:hyperlink ref="H553" r:id="GymoryHyperlink1241"/>
-    <x:hyperlink ref="J553" r:id="GymoryHyperlink1242"/>
-    <x:hyperlink ref="H554" r:id="GymoryHyperlink1243"/>
-    <x:hyperlink ref="J554" r:id="GymoryHyperlink1244"/>
-    <x:hyperlink ref="H555" r:id="GymoryHyperlink1245"/>
-    <x:hyperlink ref="J555" r:id="GymoryHyperlink1246"/>
-    <x:hyperlink ref="H556" r:id="GymoryHyperlink1247"/>
-    <x:hyperlink ref="J556" r:id="GymoryHyperlink1248"/>
-    <x:hyperlink ref="H557" r:id="GymoryHyperlink1249"/>
-    <x:hyperlink ref="J557" r:id="GymoryHyperlink1250"/>
-    <x:hyperlink ref="H558" r:id="GymoryHyperlink1251"/>
-    <x:hyperlink ref="J558" r:id="GymoryHyperlink1252"/>
-    <x:hyperlink ref="H559" r:id="GymoryHyperlink1253"/>
-    <x:hyperlink ref="J559" r:id="GymoryHyperlink1254"/>
-    <x:hyperlink ref="H560" r:id="GymoryHyperlink1255"/>
-    <x:hyperlink ref="J560" r:id="GymoryHyperlink1256"/>
-    <x:hyperlink ref="H561" r:id="GymoryHyperlink1257"/>
-    <x:hyperlink ref="J561" r:id="GymoryHyperlink1258"/>
-    <x:hyperlink ref="H562" r:id="GymoryHyperlink1259"/>
-    <x:hyperlink ref="J562" r:id="GymoryHyperlink1260"/>
-    <x:hyperlink ref="H563" r:id="GymoryHyperlink1261"/>
-    <x:hyperlink ref="J563" r:id="GymoryHyperlink1262"/>
-    <x:hyperlink ref="H564" r:id="GymoryHyperlink1263"/>
-    <x:hyperlink ref="J564" r:id="GymoryHyperlink1264"/>
-    <x:hyperlink ref="H565" r:id="GymoryHyperlink1265"/>
-    <x:hyperlink ref="J565" r:id="GymoryHyperlink1266"/>
-    <x:hyperlink ref="K565" r:id="GymoryHyperlink1267"/>
-    <x:hyperlink ref="H566" r:id="GymoryHyperlink1268"/>
-    <x:hyperlink ref="J566" r:id="GymoryHyperlink1269"/>
-    <x:hyperlink ref="K566" r:id="GymoryHyperlink1270"/>
-    <x:hyperlink ref="H567" r:id="GymoryHyperlink1271"/>
-    <x:hyperlink ref="J567" r:id="GymoryHyperlink1272"/>
-    <x:hyperlink ref="K567" r:id="GymoryHyperlink1273"/>
-    <x:hyperlink ref="H568" r:id="GymoryHyperlink1274"/>
-    <x:hyperlink ref="J568" r:id="GymoryHyperlink1275"/>
-    <x:hyperlink ref="K568" r:id="GymoryHyperlink1276"/>
-    <x:hyperlink ref="H569" r:id="GymoryHyperlink1277"/>
-    <x:hyperlink ref="J569" r:id="GymoryHyperlink1278"/>
-    <x:hyperlink ref="K569" r:id="GymoryHyperlink1279"/>
-    <x:hyperlink ref="J570" r:id="GymoryHyperlink1280"/>
-    <x:hyperlink ref="J571" r:id="GymoryHyperlink1281"/>
-    <x:hyperlink ref="J572" r:id="GymoryHyperlink1282"/>
-    <x:hyperlink ref="J573" r:id="GymoryHyperlink1283"/>
-    <x:hyperlink ref="H574" r:id="GymoryHyperlink1284"/>
-    <x:hyperlink ref="J574" r:id="GymoryHyperlink1285"/>
-    <x:hyperlink ref="H575" r:id="GymoryHyperlink1286"/>
-    <x:hyperlink ref="J575" r:id="GymoryHyperlink1287"/>
-    <x:hyperlink ref="H576" r:id="GymoryHyperlink1288"/>
-    <x:hyperlink ref="J576" r:id="GymoryHyperlink1289"/>
-    <x:hyperlink ref="H577" r:id="GymoryHyperlink1290"/>
-    <x:hyperlink ref="J577" r:id="GymoryHyperlink1291"/>
-    <x:hyperlink ref="H578" r:id="GymoryHyperlink1292"/>
-    <x:hyperlink ref="J578" r:id="GymoryHyperlink1293"/>
-    <x:hyperlink ref="H579" r:id="GymoryHyperlink1294"/>
-    <x:hyperlink ref="J579" r:id="GymoryHyperlink1295"/>
-    <x:hyperlink ref="H580" r:id="GymoryHyperlink1296"/>
-    <x:hyperlink ref="J580" r:id="GymoryHyperlink1297"/>
-    <x:hyperlink ref="H581" r:id="GymoryHyperlink1298"/>
-    <x:hyperlink ref="J581" r:id="GymoryHyperlink1299"/>
-    <x:hyperlink ref="H582" r:id="GymoryHyperlink1300"/>
-    <x:hyperlink ref="J582" r:id="GymoryHyperlink1301"/>
-    <x:hyperlink ref="H583" r:id="GymoryHyperlink1302"/>
-    <x:hyperlink ref="J583" r:id="GymoryHyperlink1303"/>
-    <x:hyperlink ref="H584" r:id="GymoryHyperlink1304"/>
-    <x:hyperlink ref="J584" r:id="GymoryHyperlink1305"/>
-    <x:hyperlink ref="H585" r:id="GymoryHyperlink1306"/>
-    <x:hyperlink ref="J585" r:id="GymoryHyperlink1307"/>
-    <x:hyperlink ref="H586" r:id="GymoryHyperlink1308"/>
-    <x:hyperlink ref="J586" r:id="GymoryHyperlink1309"/>
-    <x:hyperlink ref="H587" r:id="GymoryHyperlink1310"/>
-    <x:hyperlink ref="J587" r:id="GymoryHyperlink1311"/>
-    <x:hyperlink ref="J588" r:id="GymoryHyperlink1312"/>
-    <x:hyperlink ref="H589" r:id="GymoryHyperlink1313"/>
-    <x:hyperlink ref="J589" r:id="GymoryHyperlink1314"/>
-    <x:hyperlink ref="H590" r:id="GymoryHyperlink1315"/>
-    <x:hyperlink ref="J590" r:id="GymoryHyperlink1316"/>
-    <x:hyperlink ref="H591" r:id="GymoryHyperlink1317"/>
-    <x:hyperlink ref="J591" r:id="GymoryHyperlink1318"/>
-    <x:hyperlink ref="H592" r:id="GymoryHyperlink1319"/>
-    <x:hyperlink ref="J592" r:id="GymoryHyperlink1320"/>
-    <x:hyperlink ref="H593" r:id="GymoryHyperlink1321"/>
-    <x:hyperlink ref="J593" r:id="GymoryHyperlink1322"/>
-    <x:hyperlink ref="H594" r:id="GymoryHyperlink1323"/>
-    <x:hyperlink ref="J594" r:id="GymoryHyperlink1324"/>
-    <x:hyperlink ref="H595" r:id="GymoryHyperlink1325"/>
-    <x:hyperlink ref="J595" r:id="GymoryHyperlink1326"/>
-    <x:hyperlink ref="H596" r:id="GymoryHyperlink1327"/>
-    <x:hyperlink ref="J596" r:id="GymoryHyperlink1328"/>
-    <x:hyperlink ref="H597" r:id="GymoryHyperlink1329"/>
-    <x:hyperlink ref="J597" r:id="GymoryHyperlink1330"/>
-    <x:hyperlink ref="H598" r:id="GymoryHyperlink1331"/>
-    <x:hyperlink ref="J598" r:id="GymoryHyperlink1332"/>
-    <x:hyperlink ref="K598" r:id="GymoryHyperlink1333"/>
-    <x:hyperlink ref="H599" r:id="GymoryHyperlink1334"/>
-    <x:hyperlink ref="J599" r:id="GymoryHyperlink1335"/>
-    <x:hyperlink ref="H600" r:id="GymoryHyperlink1336"/>
-    <x:hyperlink ref="J600" r:id="GymoryHyperlink1337"/>
-    <x:hyperlink ref="H601" r:id="GymoryHyperlink1338"/>
-    <x:hyperlink ref="J601" r:id="GymoryHyperlink1339"/>
-    <x:hyperlink ref="H602" r:id="GymoryHyperlink1340"/>
-    <x:hyperlink ref="J602" r:id="GymoryHyperlink1341"/>
-    <x:hyperlink ref="H603" r:id="GymoryHyperlink1342"/>
-    <x:hyperlink ref="J603" r:id="GymoryHyperlink1343"/>
-    <x:hyperlink ref="H604" r:id="GymoryHyperlink1344"/>
-    <x:hyperlink ref="J604" r:id="GymoryHyperlink1345"/>
-    <x:hyperlink ref="H605" r:id="GymoryHyperlink1346"/>
-    <x:hyperlink ref="J605" r:id="GymoryHyperlink1347"/>
-    <x:hyperlink ref="H606" r:id="GymoryHyperlink1348"/>
-    <x:hyperlink ref="J606" r:id="GymoryHyperlink1349"/>
-    <x:hyperlink ref="H607" r:id="GymoryHyperlink1350"/>
-    <x:hyperlink ref="J607" r:id="GymoryHyperlink1351"/>
-    <x:hyperlink ref="H608" r:id="GymoryHyperlink1352"/>
-    <x:hyperlink ref="J608" r:id="GymoryHyperlink1353"/>
-    <x:hyperlink ref="H609" r:id="GymoryHyperlink1354"/>
-    <x:hyperlink ref="J609" r:id="GymoryHyperlink1355"/>
-    <x:hyperlink ref="H610" r:id="GymoryHyperlink1356"/>
-    <x:hyperlink ref="J610" r:id="GymoryHyperlink1357"/>
-    <x:hyperlink ref="H611" r:id="GymoryHyperlink1358"/>
-    <x:hyperlink ref="J611" r:id="GymoryHyperlink1359"/>
-    <x:hyperlink ref="H612" r:id="GymoryHyperlink1360"/>
-    <x:hyperlink ref="J612" r:id="GymoryHyperlink1361"/>
-    <x:hyperlink ref="H613" r:id="GymoryHyperlink1362"/>
-    <x:hyperlink ref="J613" r:id="GymoryHyperlink1363"/>
-    <x:hyperlink ref="H614" r:id="GymoryHyperlink1364"/>
-    <x:hyperlink ref="J614" r:id="GymoryHyperlink1365"/>
-    <x:hyperlink ref="H615" r:id="GymoryHyperlink1366"/>
-    <x:hyperlink ref="J615" r:id="GymoryHyperlink1367"/>
-    <x:hyperlink ref="H616" r:id="GymoryHyperlink1368"/>
-    <x:hyperlink ref="J616" r:id="GymoryHyperlink1369"/>
-    <x:hyperlink ref="H617" r:id="GymoryHyperlink1370"/>
-    <x:hyperlink ref="J617" r:id="GymoryHyperlink1371"/>
-    <x:hyperlink ref="H618" r:id="GymoryHyperlink1372"/>
-    <x:hyperlink ref="J618" r:id="GymoryHyperlink1373"/>
-    <x:hyperlink ref="H619" r:id="GymoryHyperlink1374"/>
-    <x:hyperlink ref="J619" r:id="GymoryHyperlink1375"/>
-    <x:hyperlink ref="J620" r:id="GymoryHyperlink1376"/>
-    <x:hyperlink ref="H621" r:id="GymoryHyperlink1377"/>
-    <x:hyperlink ref="J621" r:id="GymoryHyperlink1378"/>
-    <x:hyperlink ref="K621" r:id="GymoryHyperlink1379"/>
-    <x:hyperlink ref="H622" r:id="GymoryHyperlink1380"/>
-    <x:hyperlink ref="J622" r:id="GymoryHyperlink1381"/>
-    <x:hyperlink ref="J623" r:id="GymoryHyperlink1382"/>
-    <x:hyperlink ref="H624" r:id="GymoryHyperlink1383"/>
-    <x:hyperlink ref="J624" r:id="GymoryHyperlink1384"/>
-    <x:hyperlink ref="H625" r:id="GymoryHyperlink1385"/>
-    <x:hyperlink ref="J625" r:id="GymoryHyperlink1386"/>
-    <x:hyperlink ref="H626" r:id="GymoryHyperlink1387"/>
-    <x:hyperlink ref="J626" r:id="GymoryHyperlink1388"/>
-    <x:hyperlink ref="J627" r:id="GymoryHyperlink1389"/>
-    <x:hyperlink ref="K627" r:id="GymoryHyperlink1390"/>
-    <x:hyperlink ref="H628" r:id="GymoryHyperlink1391"/>
-    <x:hyperlink ref="J628" r:id="GymoryHyperlink1392"/>
-    <x:hyperlink ref="H629" r:id="GymoryHyperlink1393"/>
-    <x:hyperlink ref="J629" r:id="GymoryHyperlink1394"/>
-    <x:hyperlink ref="H630" r:id="GymoryHyperlink1395"/>
-    <x:hyperlink ref="J630" r:id="GymoryHyperlink1396"/>
-    <x:hyperlink ref="H631" r:id="GymoryHyperlink1397"/>
-    <x:hyperlink ref="J631" r:id="GymoryHyperlink1398"/>
-    <x:hyperlink ref="H632" r:id="GymoryHyperlink1399"/>
-    <x:hyperlink ref="J632" r:id="GymoryHyperlink1400"/>
-    <x:hyperlink ref="H633" r:id="GymoryHyperlink1401"/>
-    <x:hyperlink ref="J633" r:id="GymoryHyperlink1402"/>
-    <x:hyperlink ref="H634" r:id="GymoryHyperlink1403"/>
-    <x:hyperlink ref="J634" r:id="GymoryHyperlink1404"/>
-    <x:hyperlink ref="H635" r:id="GymoryHyperlink1405"/>
-    <x:hyperlink ref="J635" r:id="GymoryHyperlink1406"/>
-    <x:hyperlink ref="H636" r:id="GymoryHyperlink1407"/>
-    <x:hyperlink ref="J636" r:id="GymoryHyperlink1408"/>
-    <x:hyperlink ref="H637" r:id="GymoryHyperlink1409"/>
-    <x:hyperlink ref="J637" r:id="GymoryHyperlink1410"/>
-    <x:hyperlink ref="H638" r:id="GymoryHyperlink1411"/>
-    <x:hyperlink ref="J638" r:id="GymoryHyperlink1412"/>
-    <x:hyperlink ref="H639" r:id="GymoryHyperlink1413"/>
-    <x:hyperlink ref="J639" r:id="GymoryHyperlink1414"/>
-    <x:hyperlink ref="H640" r:id="GymoryHyperlink1415"/>
-    <x:hyperlink ref="J640" r:id="GymoryHyperlink1416"/>
-    <x:hyperlink ref="H641" r:id="GymoryHyperlink1417"/>
-    <x:hyperlink ref="J641" r:id="GymoryHyperlink1418"/>
-    <x:hyperlink ref="H642" r:id="GymoryHyperlink1419"/>
-    <x:hyperlink ref="J642" r:id="GymoryHyperlink1420"/>
-    <x:hyperlink ref="H643" r:id="GymoryHyperlink1421"/>
-    <x:hyperlink ref="J643" r:id="GymoryHyperlink1422"/>
-    <x:hyperlink ref="J644" r:id="GymoryHyperlink1423"/>
-    <x:hyperlink ref="K644" r:id="GymoryHyperlink1424"/>
-    <x:hyperlink ref="H645" r:id="GymoryHyperlink1425"/>
-    <x:hyperlink ref="J645" r:id="GymoryHyperlink1426"/>
-    <x:hyperlink ref="J646" r:id="GymoryHyperlink1427"/>
-    <x:hyperlink ref="H647" r:id="GymoryHyperlink1428"/>
-    <x:hyperlink ref="J647" r:id="GymoryHyperlink1429"/>
-    <x:hyperlink ref="J648" r:id="GymoryHyperlink1430"/>
-    <x:hyperlink ref="J649" r:id="GymoryHyperlink1431"/>
-    <x:hyperlink ref="J650" r:id="GymoryHyperlink1432"/>
-    <x:hyperlink ref="H651" r:id="GymoryHyperlink1433"/>
-    <x:hyperlink ref="J651" r:id="GymoryHyperlink1434"/>
-    <x:hyperlink ref="H652" r:id="GymoryHyperlink1435"/>
-    <x:hyperlink ref="J652" r:id="GymoryHyperlink1436"/>
-    <x:hyperlink ref="H653" r:id="GymoryHyperlink1437"/>
-    <x:hyperlink ref="J653" r:id="GymoryHyperlink1438"/>
-    <x:hyperlink ref="H654" r:id="GymoryHyperlink1439"/>
-    <x:hyperlink ref="J654" r:id="GymoryHyperlink1440"/>
-    <x:hyperlink ref="H655" r:id="GymoryHyperlink1441"/>
-    <x:hyperlink ref="J655" r:id="GymoryHyperlink1442"/>
-    <x:hyperlink ref="H656" r:id="GymoryHyperlink1443"/>
-    <x:hyperlink ref="J656" r:id="GymoryHyperlink1444"/>
-    <x:hyperlink ref="H657" r:id="GymoryHyperlink1445"/>
-    <x:hyperlink ref="J657" r:id="GymoryHyperlink1446"/>
-    <x:hyperlink ref="K657" r:id="GymoryHyperlink1447"/>
-    <x:hyperlink ref="H658" r:id="GymoryHyperlink1448"/>
-    <x:hyperlink ref="J658" r:id="GymoryHyperlink1449"/>
-    <x:hyperlink ref="J659" r:id="GymoryHyperlink1450"/>
-    <x:hyperlink ref="H660" r:id="GymoryHyperlink1451"/>
-    <x:hyperlink ref="J660" r:id="GymoryHyperlink1452"/>
-    <x:hyperlink ref="H661" r:id="GymoryHyperlink1453"/>
-    <x:hyperlink ref="J661" r:id="GymoryHyperlink1454"/>
-    <x:hyperlink ref="H662" r:id="GymoryHyperlink1455"/>
-    <x:hyperlink ref="J662" r:id="GymoryHyperlink1456"/>
-    <x:hyperlink ref="H663" r:id="GymoryHyperlink1457"/>
-    <x:hyperlink ref="J663" r:id="GymoryHyperlink1458"/>
-    <x:hyperlink ref="H664" r:id="GymoryHyperlink1459"/>
-    <x:hyperlink ref="J664" r:id="GymoryHyperlink1460"/>
-    <x:hyperlink ref="H665" r:id="GymoryHyperlink1461"/>
-    <x:hyperlink ref="J665" r:id="GymoryHyperlink1462"/>
-    <x:hyperlink ref="J666" r:id="GymoryHyperlink1463"/>
-    <x:hyperlink ref="K666" r:id="GymoryHyperlink1464"/>
-    <x:hyperlink ref="J667" r:id="GymoryHyperlink1465"/>
-    <x:hyperlink ref="J668" r:id="GymoryHyperlink1466"/>
-    <x:hyperlink ref="K668" r:id="GymoryHyperlink1467"/>
-    <x:hyperlink ref="J669" r:id="GymoryHyperlink1468"/>
-    <x:hyperlink ref="K669" r:id="GymoryHyperlink1469"/>
-    <x:hyperlink ref="J670" r:id="GymoryHyperlink1470"/>
-    <x:hyperlink ref="K670" r:id="GymoryHyperlink1471"/>
-    <x:hyperlink ref="H671" r:id="GymoryHyperlink1472"/>
-    <x:hyperlink ref="J671" r:id="GymoryHyperlink1473"/>
-    <x:hyperlink ref="J672" r:id="GymoryHyperlink1474"/>
-    <x:hyperlink ref="K672" r:id="GymoryHyperlink1475"/>
-    <x:hyperlink ref="H673" r:id="GymoryHyperlink1476"/>
-    <x:hyperlink ref="I673" r:id="GymoryHyperlink1477"/>
-    <x:hyperlink ref="J673" r:id="GymoryHyperlink1478"/>
-    <x:hyperlink ref="H674" r:id="GymoryHyperlink1479"/>
-    <x:hyperlink ref="I674" r:id="GymoryHyperlink1480"/>
-    <x:hyperlink ref="J674" r:id="GymoryHyperlink1481"/>
-    <x:hyperlink ref="H675" r:id="GymoryHyperlink1482"/>
-    <x:hyperlink ref="I675" r:id="GymoryHyperlink1483"/>
-    <x:hyperlink ref="J675" r:id="GymoryHyperlink1484"/>
-    <x:hyperlink ref="H676" r:id="GymoryHyperlink1485"/>
-    <x:hyperlink ref="I676" r:id="GymoryHyperlink1486"/>
-    <x:hyperlink ref="J676" r:id="GymoryHyperlink1487"/>
-    <x:hyperlink ref="H677" r:id="GymoryHyperlink1488"/>
-    <x:hyperlink ref="I677" r:id="GymoryHyperlink1489"/>
-    <x:hyperlink ref="J677" r:id="GymoryHyperlink1490"/>
-    <x:hyperlink ref="H678" r:id="GymoryHyperlink1491"/>
-    <x:hyperlink ref="I678" r:id="GymoryHyperlink1492"/>
-    <x:hyperlink ref="J678" r:id="GymoryHyperlink1493"/>
-    <x:hyperlink ref="H679" r:id="GymoryHyperlink1494"/>
-    <x:hyperlink ref="I679" r:id="GymoryHyperlink1495"/>
-    <x:hyperlink ref="J679" r:id="GymoryHyperlink1496"/>
-    <x:hyperlink ref="H680" r:id="GymoryHyperlink1497"/>
-    <x:hyperlink ref="I680" r:id="GymoryHyperlink1498"/>
-    <x:hyperlink ref="J680" r:id="GymoryHyperlink1499"/>
-    <x:hyperlink ref="J681" r:id="GymoryHyperlink1500"/>
-    <x:hyperlink ref="K681" r:id="GymoryHyperlink1501"/>
-    <x:hyperlink ref="J682" r:id="GymoryHyperlink1502"/>
-    <x:hyperlink ref="K682" r:id="GymoryHyperlink1503"/>
-    <x:hyperlink ref="J683" r:id="GymoryHyperlink1504"/>
-    <x:hyperlink ref="J684" r:id="GymoryHyperlink1505"/>
-    <x:hyperlink ref="J685" r:id="GymoryHyperlink1506"/>
-    <x:hyperlink ref="K685" r:id="GymoryHyperlink1507"/>
-    <x:hyperlink ref="H686" r:id="GymoryHyperlink1508"/>
-    <x:hyperlink ref="I686" r:id="GymoryHyperlink1509"/>
-    <x:hyperlink ref="J686" r:id="GymoryHyperlink1510"/>
-    <x:hyperlink ref="J687" r:id="GymoryHyperlink1511"/>
-    <x:hyperlink ref="H688" r:id="GymoryHyperlink1512"/>
-    <x:hyperlink ref="I688" r:id="GymoryHyperlink1513"/>
-    <x:hyperlink ref="J688" r:id="GymoryHyperlink1514"/>
-    <x:hyperlink ref="J689" r:id="GymoryHyperlink1515"/>
-    <x:hyperlink ref="H690" r:id="GymoryHyperlink1516"/>
-    <x:hyperlink ref="I690" r:id="GymoryHyperlink1517"/>
-    <x:hyperlink ref="J690" r:id="GymoryHyperlink1518"/>
-    <x:hyperlink ref="J691" r:id="GymoryHyperlink1519"/>
-    <x:hyperlink ref="H692" r:id="GymoryHyperlink1520"/>
-    <x:hyperlink ref="I692" r:id="GymoryHyperlink1521"/>
-    <x:hyperlink ref="J692" r:id="GymoryHyperlink1522"/>
-    <x:hyperlink ref="J693" r:id="GymoryHyperlink1523"/>
-    <x:hyperlink ref="K693" r:id="GymoryHyperlink1524"/>
-    <x:hyperlink ref="J694" r:id="GymoryHyperlink1525"/>
-    <x:hyperlink ref="K694" r:id="GymoryHyperlink1526"/>
-    <x:hyperlink ref="J695" r:id="GymoryHyperlink1527"/>
-    <x:hyperlink ref="J696" r:id="GymoryHyperlink1528"/>
-    <x:hyperlink ref="K696" r:id="GymoryHyperlink1529"/>
-    <x:hyperlink ref="J697" r:id="GymoryHyperlink1530"/>
-    <x:hyperlink ref="K697" r:id="GymoryHyperlink1531"/>
-    <x:hyperlink ref="J698" r:id="GymoryHyperlink1532"/>
-    <x:hyperlink ref="K698" r:id="GymoryHyperlink1533"/>
-    <x:hyperlink ref="J699" r:id="GymoryHyperlink1534"/>
-    <x:hyperlink ref="K699" r:id="GymoryHyperlink1535"/>
-    <x:hyperlink ref="J700" r:id="GymoryHyperlink1536"/>
-    <x:hyperlink ref="K700" r:id="GymoryHyperlink1537"/>
-    <x:hyperlink ref="J701" r:id="GymoryHyperlink1538"/>
-    <x:hyperlink ref="K701" r:id="GymoryHyperlink1539"/>
-    <x:hyperlink ref="J702" r:id="GymoryHyperlink1540"/>
-    <x:hyperlink ref="K702" r:id="GymoryHyperlink1541"/>
-    <x:hyperlink ref="J703" r:id="GymoryHyperlink1542"/>
-    <x:hyperlink ref="K703" r:id="GymoryHyperlink1543"/>
-    <x:hyperlink ref="J704" r:id="GymoryHyperlink1544"/>
-    <x:hyperlink ref="K704" r:id="GymoryHyperlink1545"/>
-    <x:hyperlink ref="J705" r:id="GymoryHyperlink1546"/>
-    <x:hyperlink ref="K705" r:id="GymoryHyperlink1547"/>
-    <x:hyperlink ref="J706" r:id="GymoryHyperlink1548"/>
-    <x:hyperlink ref="K706" r:id="GymoryHyperlink1549"/>
-    <x:hyperlink ref="J707" r:id="GymoryHyperlink1550"/>
-    <x:hyperlink ref="J708" r:id="GymoryHyperlink1551"/>
-    <x:hyperlink ref="J709" r:id="GymoryHyperlink1552"/>
-    <x:hyperlink ref="J710" r:id="GymoryHyperlink1553"/>
-    <x:hyperlink ref="H711" r:id="GymoryHyperlink1554"/>
-    <x:hyperlink ref="I711" r:id="GymoryHyperlink1555"/>
-    <x:hyperlink ref="J711" r:id="GymoryHyperlink1556"/>
-    <x:hyperlink ref="H712" r:id="GymoryHyperlink1557"/>
-    <x:hyperlink ref="I712" r:id="GymoryHyperlink1558"/>
-    <x:hyperlink ref="J712" r:id="GymoryHyperlink1559"/>
-    <x:hyperlink ref="H713" r:id="GymoryHyperlink1560"/>
-    <x:hyperlink ref="I713" r:id="GymoryHyperlink1561"/>
-    <x:hyperlink ref="J713" r:id="GymoryHyperlink1562"/>
-    <x:hyperlink ref="H714" r:id="GymoryHyperlink1563"/>
-    <x:hyperlink ref="I714" r:id="GymoryHyperlink1564"/>
-    <x:hyperlink ref="J714" r:id="GymoryHyperlink1565"/>
-    <x:hyperlink ref="H715" r:id="GymoryHyperlink1566"/>
-    <x:hyperlink ref="I715" r:id="GymoryHyperlink1567"/>
-    <x:hyperlink ref="J715" r:id="GymoryHyperlink1568"/>
-    <x:hyperlink ref="J716" r:id="GymoryHyperlink1569"/>
-    <x:hyperlink ref="K716" r:id="GymoryHyperlink1570"/>
-    <x:hyperlink ref="H717" r:id="GymoryHyperlink1571"/>
-    <x:hyperlink ref="I717" r:id="GymoryHyperlink1572"/>
-    <x:hyperlink ref="J717" r:id="GymoryHyperlink1573"/>
-    <x:hyperlink ref="H718" r:id="GymoryHyperlink1574"/>
-    <x:hyperlink ref="I718" r:id="GymoryHyperlink1575"/>
-    <x:hyperlink ref="J718" r:id="GymoryHyperlink1576"/>
-    <x:hyperlink ref="H719" r:id="GymoryHyperlink1577"/>
-    <x:hyperlink ref="I719" r:id="GymoryHyperlink1578"/>
-    <x:hyperlink ref="J719" r:id="GymoryHyperlink1579"/>
-    <x:hyperlink ref="H720" r:id="GymoryHyperlink1580"/>
-    <x:hyperlink ref="I720" r:id="GymoryHyperlink1581"/>
-    <x:hyperlink ref="J720" r:id="GymoryHyperlink1582"/>
-    <x:hyperlink ref="H721" r:id="GymoryHyperlink1583"/>
-    <x:hyperlink ref="I721" r:id="GymoryHyperlink1584"/>
-    <x:hyperlink ref="J721" r:id="GymoryHyperlink1585"/>
-    <x:hyperlink ref="H722" r:id="GymoryHyperlink1586"/>
-    <x:hyperlink ref="I722" r:id="GymoryHyperlink1587"/>
-    <x:hyperlink ref="J722" r:id="GymoryHyperlink1588"/>
-    <x:hyperlink ref="H723" r:id="GymoryHyperlink1589"/>
-    <x:hyperlink ref="I723" r:id="GymoryHyperlink1590"/>
-    <x:hyperlink ref="J723" r:id="GymoryHyperlink1591"/>
-    <x:hyperlink ref="H724" r:id="GymoryHyperlink1592"/>
-    <x:hyperlink ref="I724" r:id="GymoryHyperlink1593"/>
-    <x:hyperlink ref="J724" r:id="GymoryHyperlink1594"/>
-    <x:hyperlink ref="H725" r:id="GymoryHyperlink1595"/>
-    <x:hyperlink ref="I725" r:id="GymoryHyperlink1596"/>
-    <x:hyperlink ref="J725" r:id="GymoryHyperlink1597"/>
-    <x:hyperlink ref="H726" r:id="GymoryHyperlink1598"/>
-    <x:hyperlink ref="I726" r:id="GymoryHyperlink1599"/>
-    <x:hyperlink ref="J726" r:id="GymoryHyperlink1600"/>
-    <x:hyperlink ref="H727" r:id="GymoryHyperlink1601"/>
-    <x:hyperlink ref="I727" r:id="GymoryHyperlink1602"/>
-    <x:hyperlink ref="J727" r:id="GymoryHyperlink1603"/>
-    <x:hyperlink ref="H728" r:id="GymoryHyperlink1604"/>
-    <x:hyperlink ref="I728" r:id="GymoryHyperlink1605"/>
-    <x:hyperlink ref="J728" r:id="GymoryHyperlink1606"/>
-    <x:hyperlink ref="J729" r:id="GymoryHyperlink1607"/>
-    <x:hyperlink ref="K729" r:id="GymoryHyperlink1608"/>
-    <x:hyperlink ref="J730" r:id="GymoryHyperlink1609"/>
-    <x:hyperlink ref="K730" r:id="GymoryHyperlink1610"/>
-    <x:hyperlink ref="J731" r:id="GymoryHyperlink1611"/>
-    <x:hyperlink ref="K731" r:id="GymoryHyperlink1612"/>
-    <x:hyperlink ref="H732" r:id="GymoryHyperlink1613"/>
-    <x:hyperlink ref="I732" r:id="GymoryHyperlink1614"/>
-    <x:hyperlink ref="J732" r:id="GymoryHyperlink1615"/>
-    <x:hyperlink ref="H733" r:id="GymoryHyperlink1616"/>
-    <x:hyperlink ref="I733" r:id="GymoryHyperlink1617"/>
-    <x:hyperlink ref="J733" r:id="GymoryHyperlink1618"/>
-    <x:hyperlink ref="J734" r:id="GymoryHyperlink1619"/>
-    <x:hyperlink ref="K734" r:id="GymoryHyperlink1620"/>
-    <x:hyperlink ref="J735" r:id="GymoryHyperlink1621"/>
-    <x:hyperlink ref="K735" r:id="GymoryHyperlink1622"/>
-    <x:hyperlink ref="J736" r:id="GymoryHyperlink1623"/>
-    <x:hyperlink ref="H737" r:id="GymoryHyperlink1624"/>
-    <x:hyperlink ref="I737" r:id="GymoryHyperlink1625"/>
-    <x:hyperlink ref="J737" r:id="GymoryHyperlink1626"/>
-    <x:hyperlink ref="H738" r:id="GymoryHyperlink1627"/>
-    <x:hyperlink ref="I738" r:id="GymoryHyperlink1628"/>
-    <x:hyperlink ref="J738" r:id="GymoryHyperlink1629"/>
-    <x:hyperlink ref="H739" r:id="GymoryHyperlink1630"/>
-    <x:hyperlink ref="I739" r:id="GymoryHyperlink1631"/>
-    <x:hyperlink ref="J739" r:id="GymoryHyperlink1632"/>
-    <x:hyperlink ref="H740" r:id="GymoryHyperlink1633"/>
-    <x:hyperlink ref="I740" r:id="GymoryHyperlink1634"/>
-    <x:hyperlink ref="J740" r:id="GymoryHyperlink1635"/>
-    <x:hyperlink ref="H741" r:id="GymoryHyperlink1636"/>
-    <x:hyperlink ref="I741" r:id="GymoryHyperlink1637"/>
-    <x:hyperlink ref="J741" r:id="GymoryHyperlink1638"/>
-    <x:hyperlink ref="H742" r:id="GymoryHyperlink1639"/>
-    <x:hyperlink ref="I742" r:id="GymoryHyperlink1640"/>
-    <x:hyperlink ref="J742" r:id="GymoryHyperlink1641"/>
-    <x:hyperlink ref="H743" r:id="GymoryHyperlink1642"/>
-    <x:hyperlink ref="I743" r:id="GymoryHyperlink1643"/>
-    <x:hyperlink ref="J743" r:id="GymoryHyperlink1644"/>
-    <x:hyperlink ref="H744" r:id="GymoryHyperlink1645"/>
-    <x:hyperlink ref="I744" r:id="GymoryHyperlink1646"/>
-    <x:hyperlink ref="J744" r:id="GymoryHyperlink1647"/>
-    <x:hyperlink ref="H745" r:id="GymoryHyperlink1648"/>
-    <x:hyperlink ref="I745" r:id="GymoryHyperlink1649"/>
-    <x:hyperlink ref="J745" r:id="GymoryHyperlink1650"/>
-    <x:hyperlink ref="H746" r:id="GymoryHyperlink1651"/>
-    <x:hyperlink ref="I746" r:id="GymoryHyperlink1652"/>
-    <x:hyperlink ref="J746" r:id="GymoryHyperlink1653"/>
-    <x:hyperlink ref="H747" r:id="GymoryHyperlink1654"/>
-    <x:hyperlink ref="I747" r:id="GymoryHyperlink1655"/>
-    <x:hyperlink ref="J747" r:id="GymoryHyperlink1656"/>
-    <x:hyperlink ref="H748" r:id="GymoryHyperlink1657"/>
-    <x:hyperlink ref="I748" r:id="GymoryHyperlink1658"/>
-    <x:hyperlink ref="J748" r:id="GymoryHyperlink1659"/>
-    <x:hyperlink ref="H749" r:id="GymoryHyperlink1660"/>
-    <x:hyperlink ref="I749" r:id="GymoryHyperlink1661"/>
-    <x:hyperlink ref="J749" r:id="GymoryHyperlink1662"/>
-    <x:hyperlink ref="H750" r:id="GymoryHyperlink1663"/>
-    <x:hyperlink ref="I750" r:id="GymoryHyperlink1664"/>
-    <x:hyperlink ref="J750" r:id="GymoryHyperlink1665"/>
-    <x:hyperlink ref="H751" r:id="GymoryHyperlink1666"/>
-    <x:hyperlink ref="I751" r:id="GymoryHyperlink1667"/>
-    <x:hyperlink ref="J751" r:id="GymoryHyperlink1668"/>
-    <x:hyperlink ref="H752" r:id="GymoryHyperlink1669"/>
-    <x:hyperlink ref="I752" r:id="GymoryHyperlink1670"/>
-    <x:hyperlink ref="J752" r:id="GymoryHyperlink1671"/>
-    <x:hyperlink ref="H753" r:id="GymoryHyperlink1672"/>
-    <x:hyperlink ref="I753" r:id="GymoryHyperlink1673"/>
-    <x:hyperlink ref="J753" r:id="GymoryHyperlink1674"/>
-    <x:hyperlink ref="H754" r:id="GymoryHyperlink1675"/>
-    <x:hyperlink ref="I754" r:id="GymoryHyperlink1676"/>
-    <x:hyperlink ref="J754" r:id="GymoryHyperlink1677"/>
-    <x:hyperlink ref="H755" r:id="GymoryHyperlink1678"/>
-    <x:hyperlink ref="I755" r:id="GymoryHyperlink1679"/>
-    <x:hyperlink ref="J755" r:id="GymoryHyperlink1680"/>
-    <x:hyperlink ref="H756" r:id="GymoryHyperlink1681"/>
-    <x:hyperlink ref="I756" r:id="GymoryHyperlink1682"/>
-    <x:hyperlink ref="J756" r:id="GymoryHyperlink1683"/>
-    <x:hyperlink ref="J757" r:id="GymoryHyperlink1684"/>
-    <x:hyperlink ref="J758" r:id="GymoryHyperlink1685"/>
-    <x:hyperlink ref="J759" r:id="GymoryHyperlink1686"/>
-    <x:hyperlink ref="J760" r:id="GymoryHyperlink1687"/>
-    <x:hyperlink ref="J761" r:id="GymoryHyperlink1688"/>
-    <x:hyperlink ref="J762" r:id="GymoryHyperlink1689"/>
-    <x:hyperlink ref="K762" r:id="GymoryHyperlink1690"/>
-    <x:hyperlink ref="J763" r:id="GymoryHyperlink1691"/>
-    <x:hyperlink ref="J764" r:id="GymoryHyperlink1692"/>
-    <x:hyperlink ref="K764" r:id="GymoryHyperlink1693"/>
-    <x:hyperlink ref="J765" r:id="GymoryHyperlink1694"/>
-    <x:hyperlink ref="J766" r:id="GymoryHyperlink1695"/>
-    <x:hyperlink ref="K766" r:id="GymoryHyperlink1696"/>
-    <x:hyperlink ref="H767" r:id="GymoryHyperlink1697"/>
-    <x:hyperlink ref="I767" r:id="GymoryHyperlink1698"/>
-    <x:hyperlink ref="J767" r:id="GymoryHyperlink1699"/>
-    <x:hyperlink ref="J768" r:id="GymoryHyperlink1700"/>
-    <x:hyperlink ref="J769" r:id="GymoryHyperlink1701"/>
-    <x:hyperlink ref="J770" r:id="GymoryHyperlink1702"/>
-    <x:hyperlink ref="J771" r:id="GymoryHyperlink1703"/>
-    <x:hyperlink ref="J772" r:id="GymoryHyperlink1704"/>
-    <x:hyperlink ref="J773" r:id="GymoryHyperlink1705"/>
-    <x:hyperlink ref="J774" r:id="GymoryHyperlink1706"/>
-    <x:hyperlink ref="J775" r:id="GymoryHyperlink1707"/>
-    <x:hyperlink ref="K775" r:id="GymoryHyperlink1708"/>
-    <x:hyperlink ref="J776" r:id="GymoryHyperlink1709"/>
-    <x:hyperlink ref="J777" r:id="GymoryHyperlink1710"/>
-    <x:hyperlink ref="J778" r:id="GymoryHyperlink1711"/>
-    <x:hyperlink ref="J779" r:id="GymoryHyperlink1712"/>
-    <x:hyperlink ref="J780" r:id="GymoryHyperlink1713"/>
-    <x:hyperlink ref="J781" r:id="GymoryHyperlink1714"/>
-    <x:hyperlink ref="J782" r:id="GymoryHyperlink1715"/>
-    <x:hyperlink ref="J783" r:id="GymoryHyperlink1716"/>
-    <x:hyperlink ref="J784" r:id="GymoryHyperlink1717"/>
-    <x:hyperlink ref="J785" r:id="GymoryHyperlink1718"/>
-    <x:hyperlink ref="J786" r:id="GymoryHyperlink1719"/>
-    <x:hyperlink ref="J787" r:id="GymoryHyperlink1720"/>
-    <x:hyperlink ref="J788" r:id="GymoryHyperlink1721"/>
-    <x:hyperlink ref="J789" r:id="GymoryHyperlink1722"/>
-    <x:hyperlink ref="J790" r:id="GymoryHyperlink1723"/>
-    <x:hyperlink ref="J791" r:id="GymoryHyperlink1724"/>
-    <x:hyperlink ref="J792" r:id="GymoryHyperlink1725"/>
-    <x:hyperlink ref="J793" r:id="GymoryHyperlink1726"/>
-    <x:hyperlink ref="J794" r:id="GymoryHyperlink1727"/>
-    <x:hyperlink ref="K794" r:id="GymoryHyperlink1728"/>
-    <x:hyperlink ref="J795" r:id="GymoryHyperlink1729"/>
-    <x:hyperlink ref="J796" r:id="GymoryHyperlink1730"/>
-    <x:hyperlink ref="J797" r:id="GymoryHyperlink1731"/>
-    <x:hyperlink ref="J798" r:id="GymoryHyperlink1732"/>
-    <x:hyperlink ref="J799" r:id="GymoryHyperlink1733"/>
-    <x:hyperlink ref="J800" r:id="GymoryHyperlink1734"/>
-    <x:hyperlink ref="J801" r:id="GymoryHyperlink1735"/>
-    <x:hyperlink ref="J802" r:id="GymoryHyperlink1736"/>
-    <x:hyperlink ref="J803" r:id="GymoryHyperlink1737"/>
-    <x:hyperlink ref="J804" r:id="GymoryHyperlink1738"/>
-    <x:hyperlink ref="J805" r:id="GymoryHyperlink1739"/>
-    <x:hyperlink ref="J806" r:id="GymoryHyperlink1740"/>
-    <x:hyperlink ref="J807" r:id="GymoryHyperlink1741"/>
-    <x:hyperlink ref="K807" r:id="GymoryHyperlink1742"/>
-    <x:hyperlink ref="J808" r:id="GymoryHyperlink1743"/>
-    <x:hyperlink ref="J809" r:id="GymoryHyperlink1744"/>
-    <x:hyperlink ref="J810" r:id="GymoryHyperlink1745"/>
-    <x:hyperlink ref="J811" r:id="GymoryHyperlink1746"/>
-    <x:hyperlink ref="J812" r:id="GymoryHyperlink1747"/>
-    <x:hyperlink ref="J813" r:id="GymoryHyperlink1748"/>
-    <x:hyperlink ref="J814" r:id="GymoryHyperlink1749"/>
-    <x:hyperlink ref="J815" r:id="GymoryHyperlink1750"/>
-    <x:hyperlink ref="J816" r:id="GymoryHyperlink1751"/>
-    <x:hyperlink ref="J817" r:id="GymoryHyperlink1752"/>
-    <x:hyperlink ref="J818" r:id="GymoryHyperlink1753"/>
-    <x:hyperlink ref="J819" r:id="GymoryHyperlink1754"/>
-    <x:hyperlink ref="J820" r:id="GymoryHyperlink1755"/>
-    <x:hyperlink ref="J821" r:id="GymoryHyperlink1756"/>
-    <x:hyperlink ref="J822" r:id="GymoryHyperlink1757"/>
-    <x:hyperlink ref="J823" r:id="GymoryHyperlink1758"/>
-    <x:hyperlink ref="J824" r:id="GymoryHyperlink1759"/>
-    <x:hyperlink ref="J825" r:id="GymoryHyperlink1760"/>
-    <x:hyperlink ref="J826" r:id="GymoryHyperlink1761"/>
-    <x:hyperlink ref="J827" r:id="GymoryHyperlink1762"/>
-    <x:hyperlink ref="K827" r:id="GymoryHyperlink1763"/>
-    <x:hyperlink ref="J828" r:id="GymoryHyperlink1764"/>
-    <x:hyperlink ref="J829" r:id="GymoryHyperlink1765"/>
-    <x:hyperlink ref="J830" r:id="GymoryHyperlink1766"/>
-    <x:hyperlink ref="J831" r:id="GymoryHyperlink1767"/>
-    <x:hyperlink ref="J832" r:id="GymoryHyperlink1768"/>
-    <x:hyperlink ref="K832" r:id="GymoryHyperlink1769"/>
-    <x:hyperlink ref="J833" r:id="GymoryHyperlink1770"/>
-    <x:hyperlink ref="K833" r:id="GymoryHyperlink1771"/>
-    <x:hyperlink ref="J834" r:id="GymoryHyperlink1772"/>
-    <x:hyperlink ref="J835" r:id="GymoryHyperlink1773"/>
-    <x:hyperlink ref="K835" r:id="GymoryHyperlink1774"/>
-    <x:hyperlink ref="J836" r:id="GymoryHyperlink1775"/>
-    <x:hyperlink ref="K836" r:id="GymoryHyperlink1776"/>
-    <x:hyperlink ref="J837" r:id="GymoryHyperlink1777"/>
-    <x:hyperlink ref="K837" r:id="GymoryHyperlink1778"/>
+    <x:hyperlink ref="H497" r:id="GymoryHyperlink1130"/>
+    <x:hyperlink ref="I497" r:id="GymoryHyperlink1131"/>
+    <x:hyperlink ref="J497" r:id="GymoryHyperlink1132"/>
+    <x:hyperlink ref="H498" r:id="GymoryHyperlink1133"/>
+    <x:hyperlink ref="I498" r:id="GymoryHyperlink1134"/>
+    <x:hyperlink ref="J498" r:id="GymoryHyperlink1135"/>
+    <x:hyperlink ref="H499" r:id="GymoryHyperlink1136"/>
+    <x:hyperlink ref="I499" r:id="GymoryHyperlink1137"/>
+    <x:hyperlink ref="J499" r:id="GymoryHyperlink1138"/>
+    <x:hyperlink ref="H500" r:id="GymoryHyperlink1139"/>
+    <x:hyperlink ref="I500" r:id="GymoryHyperlink1140"/>
+    <x:hyperlink ref="J500" r:id="GymoryHyperlink1141"/>
+    <x:hyperlink ref="H501" r:id="GymoryHyperlink1142"/>
+    <x:hyperlink ref="I501" r:id="GymoryHyperlink1143"/>
+    <x:hyperlink ref="J501" r:id="GymoryHyperlink1144"/>
+    <x:hyperlink ref="H502" r:id="GymoryHyperlink1145"/>
+    <x:hyperlink ref="I502" r:id="GymoryHyperlink1146"/>
+    <x:hyperlink ref="J502" r:id="GymoryHyperlink1147"/>
+    <x:hyperlink ref="H503" r:id="GymoryHyperlink1148"/>
+    <x:hyperlink ref="I503" r:id="GymoryHyperlink1149"/>
+    <x:hyperlink ref="J503" r:id="GymoryHyperlink1150"/>
+    <x:hyperlink ref="H504" r:id="GymoryHyperlink1151"/>
+    <x:hyperlink ref="I504" r:id="GymoryHyperlink1152"/>
+    <x:hyperlink ref="J504" r:id="GymoryHyperlink1153"/>
+    <x:hyperlink ref="H505" r:id="GymoryHyperlink1154"/>
+    <x:hyperlink ref="I505" r:id="GymoryHyperlink1155"/>
+    <x:hyperlink ref="J505" r:id="GymoryHyperlink1156"/>
+    <x:hyperlink ref="H506" r:id="GymoryHyperlink1157"/>
+    <x:hyperlink ref="I506" r:id="GymoryHyperlink1158"/>
+    <x:hyperlink ref="J506" r:id="GymoryHyperlink1159"/>
+    <x:hyperlink ref="H507" r:id="GymoryHyperlink1160"/>
+    <x:hyperlink ref="I507" r:id="GymoryHyperlink1161"/>
+    <x:hyperlink ref="J507" r:id="GymoryHyperlink1162"/>
+    <x:hyperlink ref="H508" r:id="GymoryHyperlink1163"/>
+    <x:hyperlink ref="I508" r:id="GymoryHyperlink1164"/>
+    <x:hyperlink ref="J508" r:id="GymoryHyperlink1165"/>
+    <x:hyperlink ref="H509" r:id="GymoryHyperlink1166"/>
+    <x:hyperlink ref="I509" r:id="GymoryHyperlink1167"/>
+    <x:hyperlink ref="J509" r:id="GymoryHyperlink1168"/>
+    <x:hyperlink ref="H510" r:id="GymoryHyperlink1169"/>
+    <x:hyperlink ref="I510" r:id="GymoryHyperlink1170"/>
+    <x:hyperlink ref="J510" r:id="GymoryHyperlink1171"/>
+    <x:hyperlink ref="H511" r:id="GymoryHyperlink1172"/>
+    <x:hyperlink ref="I511" r:id="GymoryHyperlink1173"/>
+    <x:hyperlink ref="J511" r:id="GymoryHyperlink1174"/>
+    <x:hyperlink ref="H512" r:id="GymoryHyperlink1175"/>
+    <x:hyperlink ref="I512" r:id="GymoryHyperlink1176"/>
+    <x:hyperlink ref="J512" r:id="GymoryHyperlink1177"/>
+    <x:hyperlink ref="H513" r:id="GymoryHyperlink1178"/>
+    <x:hyperlink ref="I513" r:id="GymoryHyperlink1179"/>
+    <x:hyperlink ref="J513" r:id="GymoryHyperlink1180"/>
+    <x:hyperlink ref="H514" r:id="GymoryHyperlink1181"/>
+    <x:hyperlink ref="I514" r:id="GymoryHyperlink1182"/>
+    <x:hyperlink ref="J514" r:id="GymoryHyperlink1183"/>
+    <x:hyperlink ref="H515" r:id="GymoryHyperlink1184"/>
+    <x:hyperlink ref="I515" r:id="GymoryHyperlink1185"/>
+    <x:hyperlink ref="J515" r:id="GymoryHyperlink1186"/>
+    <x:hyperlink ref="H516" r:id="GymoryHyperlink1187"/>
+    <x:hyperlink ref="I516" r:id="GymoryHyperlink1188"/>
+    <x:hyperlink ref="J516" r:id="GymoryHyperlink1189"/>
+    <x:hyperlink ref="H517" r:id="GymoryHyperlink1190"/>
+    <x:hyperlink ref="I517" r:id="GymoryHyperlink1191"/>
+    <x:hyperlink ref="J517" r:id="GymoryHyperlink1192"/>
+    <x:hyperlink ref="H518" r:id="GymoryHyperlink1193"/>
+    <x:hyperlink ref="I518" r:id="GymoryHyperlink1194"/>
+    <x:hyperlink ref="J518" r:id="GymoryHyperlink1195"/>
+    <x:hyperlink ref="H519" r:id="GymoryHyperlink1196"/>
+    <x:hyperlink ref="I519" r:id="GymoryHyperlink1197"/>
+    <x:hyperlink ref="J519" r:id="GymoryHyperlink1198"/>
+    <x:hyperlink ref="H520" r:id="GymoryHyperlink1199"/>
+    <x:hyperlink ref="I520" r:id="GymoryHyperlink1200"/>
+    <x:hyperlink ref="J520" r:id="GymoryHyperlink1201"/>
+    <x:hyperlink ref="H521" r:id="GymoryHyperlink1202"/>
+    <x:hyperlink ref="I521" r:id="GymoryHyperlink1203"/>
+    <x:hyperlink ref="J521" r:id="GymoryHyperlink1204"/>
+    <x:hyperlink ref="H522" r:id="GymoryHyperlink1205"/>
+    <x:hyperlink ref="I522" r:id="GymoryHyperlink1206"/>
+    <x:hyperlink ref="J522" r:id="GymoryHyperlink1207"/>
+    <x:hyperlink ref="H523" r:id="GymoryHyperlink1208"/>
+    <x:hyperlink ref="I523" r:id="GymoryHyperlink1209"/>
+    <x:hyperlink ref="J523" r:id="GymoryHyperlink1210"/>
+    <x:hyperlink ref="H524" r:id="GymoryHyperlink1211"/>
+    <x:hyperlink ref="I524" r:id="GymoryHyperlink1212"/>
+    <x:hyperlink ref="J524" r:id="GymoryHyperlink1213"/>
+    <x:hyperlink ref="H525" r:id="GymoryHyperlink1214"/>
+    <x:hyperlink ref="I525" r:id="GymoryHyperlink1215"/>
+    <x:hyperlink ref="J525" r:id="GymoryHyperlink1216"/>
+    <x:hyperlink ref="H526" r:id="GymoryHyperlink1217"/>
+    <x:hyperlink ref="I526" r:id="GymoryHyperlink1218"/>
+    <x:hyperlink ref="J526" r:id="GymoryHyperlink1219"/>
+    <x:hyperlink ref="H527" r:id="GymoryHyperlink1220"/>
+    <x:hyperlink ref="I527" r:id="GymoryHyperlink1221"/>
+    <x:hyperlink ref="J527" r:id="GymoryHyperlink1222"/>
+    <x:hyperlink ref="H528" r:id="GymoryHyperlink1223"/>
+    <x:hyperlink ref="I528" r:id="GymoryHyperlink1224"/>
+    <x:hyperlink ref="J528" r:id="GymoryHyperlink1225"/>
+    <x:hyperlink ref="H529" r:id="GymoryHyperlink1226"/>
+    <x:hyperlink ref="I529" r:id="GymoryHyperlink1227"/>
+    <x:hyperlink ref="J529" r:id="GymoryHyperlink1228"/>
+    <x:hyperlink ref="H530" r:id="GymoryHyperlink1229"/>
+    <x:hyperlink ref="I530" r:id="GymoryHyperlink1230"/>
+    <x:hyperlink ref="J530" r:id="GymoryHyperlink1231"/>
+    <x:hyperlink ref="H531" r:id="GymoryHyperlink1232"/>
+    <x:hyperlink ref="I531" r:id="GymoryHyperlink1233"/>
+    <x:hyperlink ref="J531" r:id="GymoryHyperlink1234"/>
+    <x:hyperlink ref="H532" r:id="GymoryHyperlink1235"/>
+    <x:hyperlink ref="I532" r:id="GymoryHyperlink1236"/>
+    <x:hyperlink ref="J532" r:id="GymoryHyperlink1237"/>
+    <x:hyperlink ref="H533" r:id="GymoryHyperlink1238"/>
+    <x:hyperlink ref="I533" r:id="GymoryHyperlink1239"/>
+    <x:hyperlink ref="J533" r:id="GymoryHyperlink1240"/>
+    <x:hyperlink ref="H534" r:id="GymoryHyperlink1241"/>
+    <x:hyperlink ref="I534" r:id="GymoryHyperlink1242"/>
+    <x:hyperlink ref="J534" r:id="GymoryHyperlink1243"/>
+    <x:hyperlink ref="H535" r:id="GymoryHyperlink1244"/>
+    <x:hyperlink ref="I535" r:id="GymoryHyperlink1245"/>
+    <x:hyperlink ref="J535" r:id="GymoryHyperlink1246"/>
+    <x:hyperlink ref="H536" r:id="GymoryHyperlink1247"/>
+    <x:hyperlink ref="I536" r:id="GymoryHyperlink1248"/>
+    <x:hyperlink ref="J536" r:id="GymoryHyperlink1249"/>
+    <x:hyperlink ref="H537" r:id="GymoryHyperlink1250"/>
+    <x:hyperlink ref="I537" r:id="GymoryHyperlink1251"/>
+    <x:hyperlink ref="J537" r:id="GymoryHyperlink1252"/>
+    <x:hyperlink ref="H538" r:id="GymoryHyperlink1253"/>
+    <x:hyperlink ref="I538" r:id="GymoryHyperlink1254"/>
+    <x:hyperlink ref="J538" r:id="GymoryHyperlink1255"/>
+    <x:hyperlink ref="H539" r:id="GymoryHyperlink1256"/>
+    <x:hyperlink ref="I539" r:id="GymoryHyperlink1257"/>
+    <x:hyperlink ref="J539" r:id="GymoryHyperlink1258"/>
+    <x:hyperlink ref="H540" r:id="GymoryHyperlink1259"/>
+    <x:hyperlink ref="I540" r:id="GymoryHyperlink1260"/>
+    <x:hyperlink ref="J540" r:id="GymoryHyperlink1261"/>
+    <x:hyperlink ref="H541" r:id="GymoryHyperlink1262"/>
+    <x:hyperlink ref="I541" r:id="GymoryHyperlink1263"/>
+    <x:hyperlink ref="J541" r:id="GymoryHyperlink1264"/>
+    <x:hyperlink ref="H542" r:id="GymoryHyperlink1265"/>
+    <x:hyperlink ref="I542" r:id="GymoryHyperlink1266"/>
+    <x:hyperlink ref="J542" r:id="GymoryHyperlink1267"/>
+    <x:hyperlink ref="H543" r:id="GymoryHyperlink1268"/>
+    <x:hyperlink ref="I543" r:id="GymoryHyperlink1269"/>
+    <x:hyperlink ref="J543" r:id="GymoryHyperlink1270"/>
+    <x:hyperlink ref="H544" r:id="GymoryHyperlink1271"/>
+    <x:hyperlink ref="I544" r:id="GymoryHyperlink1272"/>
+    <x:hyperlink ref="J544" r:id="GymoryHyperlink1273"/>
+    <x:hyperlink ref="H545" r:id="GymoryHyperlink1274"/>
+    <x:hyperlink ref="I545" r:id="GymoryHyperlink1275"/>
+    <x:hyperlink ref="J545" r:id="GymoryHyperlink1276"/>
+    <x:hyperlink ref="H546" r:id="GymoryHyperlink1277"/>
+    <x:hyperlink ref="I546" r:id="GymoryHyperlink1278"/>
+    <x:hyperlink ref="J546" r:id="GymoryHyperlink1279"/>
+    <x:hyperlink ref="H547" r:id="GymoryHyperlink1280"/>
+    <x:hyperlink ref="I547" r:id="GymoryHyperlink1281"/>
+    <x:hyperlink ref="J547" r:id="GymoryHyperlink1282"/>
+    <x:hyperlink ref="H548" r:id="GymoryHyperlink1283"/>
+    <x:hyperlink ref="I548" r:id="GymoryHyperlink1284"/>
+    <x:hyperlink ref="J548" r:id="GymoryHyperlink1285"/>
+    <x:hyperlink ref="H549" r:id="GymoryHyperlink1286"/>
+    <x:hyperlink ref="I549" r:id="GymoryHyperlink1287"/>
+    <x:hyperlink ref="J549" r:id="GymoryHyperlink1288"/>
+    <x:hyperlink ref="H550" r:id="GymoryHyperlink1289"/>
+    <x:hyperlink ref="I550" r:id="GymoryHyperlink1290"/>
+    <x:hyperlink ref="J550" r:id="GymoryHyperlink1291"/>
+    <x:hyperlink ref="H551" r:id="GymoryHyperlink1292"/>
+    <x:hyperlink ref="I551" r:id="GymoryHyperlink1293"/>
+    <x:hyperlink ref="J551" r:id="GymoryHyperlink1294"/>
+    <x:hyperlink ref="H552" r:id="GymoryHyperlink1295"/>
+    <x:hyperlink ref="I552" r:id="GymoryHyperlink1296"/>
+    <x:hyperlink ref="J552" r:id="GymoryHyperlink1297"/>
+    <x:hyperlink ref="H553" r:id="GymoryHyperlink1298"/>
+    <x:hyperlink ref="I553" r:id="GymoryHyperlink1299"/>
+    <x:hyperlink ref="J553" r:id="GymoryHyperlink1300"/>
+    <x:hyperlink ref="H554" r:id="GymoryHyperlink1301"/>
+    <x:hyperlink ref="I554" r:id="GymoryHyperlink1302"/>
+    <x:hyperlink ref="J554" r:id="GymoryHyperlink1303"/>
+    <x:hyperlink ref="H555" r:id="GymoryHyperlink1304"/>
+    <x:hyperlink ref="I555" r:id="GymoryHyperlink1305"/>
+    <x:hyperlink ref="J555" r:id="GymoryHyperlink1306"/>
+    <x:hyperlink ref="H556" r:id="GymoryHyperlink1307"/>
+    <x:hyperlink ref="I556" r:id="GymoryHyperlink1308"/>
+    <x:hyperlink ref="J556" r:id="GymoryHyperlink1309"/>
+    <x:hyperlink ref="H557" r:id="GymoryHyperlink1310"/>
+    <x:hyperlink ref="I557" r:id="GymoryHyperlink1311"/>
+    <x:hyperlink ref="J557" r:id="GymoryHyperlink1312"/>
+    <x:hyperlink ref="H558" r:id="GymoryHyperlink1313"/>
+    <x:hyperlink ref="I558" r:id="GymoryHyperlink1314"/>
+    <x:hyperlink ref="J558" r:id="GymoryHyperlink1315"/>
+    <x:hyperlink ref="H559" r:id="GymoryHyperlink1316"/>
+    <x:hyperlink ref="I559" r:id="GymoryHyperlink1317"/>
+    <x:hyperlink ref="J559" r:id="GymoryHyperlink1318"/>
+    <x:hyperlink ref="H560" r:id="GymoryHyperlink1319"/>
+    <x:hyperlink ref="I560" r:id="GymoryHyperlink1320"/>
+    <x:hyperlink ref="J560" r:id="GymoryHyperlink1321"/>
+    <x:hyperlink ref="H561" r:id="GymoryHyperlink1322"/>
+    <x:hyperlink ref="I561" r:id="GymoryHyperlink1323"/>
+    <x:hyperlink ref="J561" r:id="GymoryHyperlink1324"/>
+    <x:hyperlink ref="H562" r:id="GymoryHyperlink1325"/>
+    <x:hyperlink ref="I562" r:id="GymoryHyperlink1326"/>
+    <x:hyperlink ref="J562" r:id="GymoryHyperlink1327"/>
+    <x:hyperlink ref="H563" r:id="GymoryHyperlink1328"/>
+    <x:hyperlink ref="I563" r:id="GymoryHyperlink1329"/>
+    <x:hyperlink ref="J563" r:id="GymoryHyperlink1330"/>
+    <x:hyperlink ref="H564" r:id="GymoryHyperlink1331"/>
+    <x:hyperlink ref="I564" r:id="GymoryHyperlink1332"/>
+    <x:hyperlink ref="J564" r:id="GymoryHyperlink1333"/>
+    <x:hyperlink ref="H565" r:id="GymoryHyperlink1334"/>
+    <x:hyperlink ref="I565" r:id="GymoryHyperlink1335"/>
+    <x:hyperlink ref="J565" r:id="GymoryHyperlink1336"/>
+    <x:hyperlink ref="H566" r:id="GymoryHyperlink1337"/>
+    <x:hyperlink ref="I566" r:id="GymoryHyperlink1338"/>
+    <x:hyperlink ref="J566" r:id="GymoryHyperlink1339"/>
+    <x:hyperlink ref="H567" r:id="GymoryHyperlink1340"/>
+    <x:hyperlink ref="I567" r:id="GymoryHyperlink1341"/>
+    <x:hyperlink ref="J567" r:id="GymoryHyperlink1342"/>
+    <x:hyperlink ref="H568" r:id="GymoryHyperlink1343"/>
+    <x:hyperlink ref="I568" r:id="GymoryHyperlink1344"/>
+    <x:hyperlink ref="J568" r:id="GymoryHyperlink1345"/>
+    <x:hyperlink ref="H569" r:id="GymoryHyperlink1346"/>
+    <x:hyperlink ref="I569" r:id="GymoryHyperlink1347"/>
+    <x:hyperlink ref="J569" r:id="GymoryHyperlink1348"/>
+    <x:hyperlink ref="H570" r:id="GymoryHyperlink1349"/>
+    <x:hyperlink ref="I570" r:id="GymoryHyperlink1350"/>
+    <x:hyperlink ref="J570" r:id="GymoryHyperlink1351"/>
+    <x:hyperlink ref="H571" r:id="GymoryHyperlink1352"/>
+    <x:hyperlink ref="I571" r:id="GymoryHyperlink1353"/>
+    <x:hyperlink ref="J571" r:id="GymoryHyperlink1354"/>
+    <x:hyperlink ref="H572" r:id="GymoryHyperlink1355"/>
+    <x:hyperlink ref="I572" r:id="GymoryHyperlink1356"/>
+    <x:hyperlink ref="J572" r:id="GymoryHyperlink1357"/>
+    <x:hyperlink ref="H573" r:id="GymoryHyperlink1358"/>
+    <x:hyperlink ref="I573" r:id="GymoryHyperlink1359"/>
+    <x:hyperlink ref="J573" r:id="GymoryHyperlink1360"/>
+    <x:hyperlink ref="H574" r:id="GymoryHyperlink1361"/>
+    <x:hyperlink ref="I574" r:id="GymoryHyperlink1362"/>
+    <x:hyperlink ref="J574" r:id="GymoryHyperlink1363"/>
+    <x:hyperlink ref="H575" r:id="GymoryHyperlink1364"/>
+    <x:hyperlink ref="I575" r:id="GymoryHyperlink1365"/>
+    <x:hyperlink ref="J575" r:id="GymoryHyperlink1366"/>
+    <x:hyperlink ref="H576" r:id="GymoryHyperlink1367"/>
+    <x:hyperlink ref="I576" r:id="GymoryHyperlink1368"/>
+    <x:hyperlink ref="J576" r:id="GymoryHyperlink1369"/>
+    <x:hyperlink ref="H577" r:id="GymoryHyperlink1370"/>
+    <x:hyperlink ref="I577" r:id="GymoryHyperlink1371"/>
+    <x:hyperlink ref="J577" r:id="GymoryHyperlink1372"/>
+    <x:hyperlink ref="H578" r:id="GymoryHyperlink1373"/>
+    <x:hyperlink ref="I578" r:id="GymoryHyperlink1374"/>
+    <x:hyperlink ref="J578" r:id="GymoryHyperlink1375"/>
+    <x:hyperlink ref="H579" r:id="GymoryHyperlink1376"/>
+    <x:hyperlink ref="I579" r:id="GymoryHyperlink1377"/>
+    <x:hyperlink ref="J579" r:id="GymoryHyperlink1378"/>
+    <x:hyperlink ref="H580" r:id="GymoryHyperlink1379"/>
+    <x:hyperlink ref="I580" r:id="GymoryHyperlink1380"/>
+    <x:hyperlink ref="J580" r:id="GymoryHyperlink1381"/>
+    <x:hyperlink ref="H581" r:id="GymoryHyperlink1382"/>
+    <x:hyperlink ref="I581" r:id="GymoryHyperlink1383"/>
+    <x:hyperlink ref="J581" r:id="GymoryHyperlink1384"/>
+    <x:hyperlink ref="H582" r:id="GymoryHyperlink1385"/>
+    <x:hyperlink ref="I582" r:id="GymoryHyperlink1386"/>
+    <x:hyperlink ref="J582" r:id="GymoryHyperlink1387"/>
+    <x:hyperlink ref="H583" r:id="GymoryHyperlink1388"/>
+    <x:hyperlink ref="I583" r:id="GymoryHyperlink1389"/>
+    <x:hyperlink ref="J583" r:id="GymoryHyperlink1390"/>
+    <x:hyperlink ref="H584" r:id="GymoryHyperlink1391"/>
+    <x:hyperlink ref="I584" r:id="GymoryHyperlink1392"/>
+    <x:hyperlink ref="J584" r:id="GymoryHyperlink1393"/>
+    <x:hyperlink ref="H585" r:id="GymoryHyperlink1394"/>
+    <x:hyperlink ref="I585" r:id="GymoryHyperlink1395"/>
+    <x:hyperlink ref="J585" r:id="GymoryHyperlink1396"/>
+    <x:hyperlink ref="H586" r:id="GymoryHyperlink1397"/>
+    <x:hyperlink ref="I586" r:id="GymoryHyperlink1398"/>
+    <x:hyperlink ref="J586" r:id="GymoryHyperlink1399"/>
+    <x:hyperlink ref="H587" r:id="GymoryHyperlink1400"/>
+    <x:hyperlink ref="I587" r:id="GymoryHyperlink1401"/>
+    <x:hyperlink ref="J587" r:id="GymoryHyperlink1402"/>
+    <x:hyperlink ref="J588" r:id="GymoryHyperlink1403"/>
+    <x:hyperlink ref="H589" r:id="GymoryHyperlink1404"/>
+    <x:hyperlink ref="I589" r:id="GymoryHyperlink1405"/>
+    <x:hyperlink ref="J589" r:id="GymoryHyperlink1406"/>
+    <x:hyperlink ref="H590" r:id="GymoryHyperlink1407"/>
+    <x:hyperlink ref="I590" r:id="GymoryHyperlink1408"/>
+    <x:hyperlink ref="J590" r:id="GymoryHyperlink1409"/>
+    <x:hyperlink ref="H591" r:id="GymoryHyperlink1410"/>
+    <x:hyperlink ref="I591" r:id="GymoryHyperlink1411"/>
+    <x:hyperlink ref="J591" r:id="GymoryHyperlink1412"/>
+    <x:hyperlink ref="H592" r:id="GymoryHyperlink1413"/>
+    <x:hyperlink ref="I592" r:id="GymoryHyperlink1414"/>
+    <x:hyperlink ref="J592" r:id="GymoryHyperlink1415"/>
+    <x:hyperlink ref="H593" r:id="GymoryHyperlink1416"/>
+    <x:hyperlink ref="I593" r:id="GymoryHyperlink1417"/>
+    <x:hyperlink ref="J593" r:id="GymoryHyperlink1418"/>
+    <x:hyperlink ref="H594" r:id="GymoryHyperlink1419"/>
+    <x:hyperlink ref="I594" r:id="GymoryHyperlink1420"/>
+    <x:hyperlink ref="J594" r:id="GymoryHyperlink1421"/>
+    <x:hyperlink ref="H595" r:id="GymoryHyperlink1422"/>
+    <x:hyperlink ref="I595" r:id="GymoryHyperlink1423"/>
+    <x:hyperlink ref="J595" r:id="GymoryHyperlink1424"/>
+    <x:hyperlink ref="H596" r:id="GymoryHyperlink1425"/>
+    <x:hyperlink ref="I596" r:id="GymoryHyperlink1426"/>
+    <x:hyperlink ref="J596" r:id="GymoryHyperlink1427"/>
+    <x:hyperlink ref="H597" r:id="GymoryHyperlink1428"/>
+    <x:hyperlink ref="I597" r:id="GymoryHyperlink1429"/>
+    <x:hyperlink ref="J597" r:id="GymoryHyperlink1430"/>
+    <x:hyperlink ref="H598" r:id="GymoryHyperlink1431"/>
+    <x:hyperlink ref="I598" r:id="GymoryHyperlink1432"/>
+    <x:hyperlink ref="J598" r:id="GymoryHyperlink1433"/>
+    <x:hyperlink ref="H599" r:id="GymoryHyperlink1434"/>
+    <x:hyperlink ref="I599" r:id="GymoryHyperlink1435"/>
+    <x:hyperlink ref="J599" r:id="GymoryHyperlink1436"/>
+    <x:hyperlink ref="H600" r:id="GymoryHyperlink1437"/>
+    <x:hyperlink ref="I600" r:id="GymoryHyperlink1438"/>
+    <x:hyperlink ref="J600" r:id="GymoryHyperlink1439"/>
+    <x:hyperlink ref="H601" r:id="GymoryHyperlink1440"/>
+    <x:hyperlink ref="I601" r:id="GymoryHyperlink1441"/>
+    <x:hyperlink ref="J601" r:id="GymoryHyperlink1442"/>
+    <x:hyperlink ref="H602" r:id="GymoryHyperlink1443"/>
+    <x:hyperlink ref="I602" r:id="GymoryHyperlink1444"/>
+    <x:hyperlink ref="J602" r:id="GymoryHyperlink1445"/>
+    <x:hyperlink ref="H603" r:id="GymoryHyperlink1446"/>
+    <x:hyperlink ref="I603" r:id="GymoryHyperlink1447"/>
+    <x:hyperlink ref="J603" r:id="GymoryHyperlink1448"/>
+    <x:hyperlink ref="H604" r:id="GymoryHyperlink1449"/>
+    <x:hyperlink ref="I604" r:id="GymoryHyperlink1450"/>
+    <x:hyperlink ref="J604" r:id="GymoryHyperlink1451"/>
+    <x:hyperlink ref="H605" r:id="GymoryHyperlink1452"/>
+    <x:hyperlink ref="I605" r:id="GymoryHyperlink1453"/>
+    <x:hyperlink ref="J605" r:id="GymoryHyperlink1454"/>
+    <x:hyperlink ref="H606" r:id="GymoryHyperlink1455"/>
+    <x:hyperlink ref="I606" r:id="GymoryHyperlink1456"/>
+    <x:hyperlink ref="J606" r:id="GymoryHyperlink1457"/>
+    <x:hyperlink ref="H607" r:id="GymoryHyperlink1458"/>
+    <x:hyperlink ref="I607" r:id="GymoryHyperlink1459"/>
+    <x:hyperlink ref="J607" r:id="GymoryHyperlink1460"/>
+    <x:hyperlink ref="H608" r:id="GymoryHyperlink1461"/>
+    <x:hyperlink ref="I608" r:id="GymoryHyperlink1462"/>
+    <x:hyperlink ref="J608" r:id="GymoryHyperlink1463"/>
+    <x:hyperlink ref="H609" r:id="GymoryHyperlink1464"/>
+    <x:hyperlink ref="I609" r:id="GymoryHyperlink1465"/>
+    <x:hyperlink ref="J609" r:id="GymoryHyperlink1466"/>
+    <x:hyperlink ref="H610" r:id="GymoryHyperlink1467"/>
+    <x:hyperlink ref="I610" r:id="GymoryHyperlink1468"/>
+    <x:hyperlink ref="J610" r:id="GymoryHyperlink1469"/>
+    <x:hyperlink ref="H611" r:id="GymoryHyperlink1470"/>
+    <x:hyperlink ref="I611" r:id="GymoryHyperlink1471"/>
+    <x:hyperlink ref="J611" r:id="GymoryHyperlink1472"/>
+    <x:hyperlink ref="H612" r:id="GymoryHyperlink1473"/>
+    <x:hyperlink ref="I612" r:id="GymoryHyperlink1474"/>
+    <x:hyperlink ref="J612" r:id="GymoryHyperlink1475"/>
+    <x:hyperlink ref="H613" r:id="GymoryHyperlink1476"/>
+    <x:hyperlink ref="I613" r:id="GymoryHyperlink1477"/>
+    <x:hyperlink ref="J613" r:id="GymoryHyperlink1478"/>
+    <x:hyperlink ref="H614" r:id="GymoryHyperlink1479"/>
+    <x:hyperlink ref="I614" r:id="GymoryHyperlink1480"/>
+    <x:hyperlink ref="J614" r:id="GymoryHyperlink1481"/>
+    <x:hyperlink ref="H615" r:id="GymoryHyperlink1482"/>
+    <x:hyperlink ref="I615" r:id="GymoryHyperlink1483"/>
+    <x:hyperlink ref="J615" r:id="GymoryHyperlink1484"/>
+    <x:hyperlink ref="H616" r:id="GymoryHyperlink1485"/>
+    <x:hyperlink ref="I616" r:id="GymoryHyperlink1486"/>
+    <x:hyperlink ref="J616" r:id="GymoryHyperlink1487"/>
+    <x:hyperlink ref="H617" r:id="GymoryHyperlink1488"/>
+    <x:hyperlink ref="I617" r:id="GymoryHyperlink1489"/>
+    <x:hyperlink ref="J617" r:id="GymoryHyperlink1490"/>
+    <x:hyperlink ref="H618" r:id="GymoryHyperlink1491"/>
+    <x:hyperlink ref="I618" r:id="GymoryHyperlink1492"/>
+    <x:hyperlink ref="J618" r:id="GymoryHyperlink1493"/>
+    <x:hyperlink ref="H619" r:id="GymoryHyperlink1494"/>
+    <x:hyperlink ref="I619" r:id="GymoryHyperlink1495"/>
+    <x:hyperlink ref="J619" r:id="GymoryHyperlink1496"/>
+    <x:hyperlink ref="H620" r:id="GymoryHyperlink1497"/>
+    <x:hyperlink ref="I620" r:id="GymoryHyperlink1498"/>
+    <x:hyperlink ref="J620" r:id="GymoryHyperlink1499"/>
+    <x:hyperlink ref="H621" r:id="GymoryHyperlink1500"/>
+    <x:hyperlink ref="I621" r:id="GymoryHyperlink1501"/>
+    <x:hyperlink ref="J621" r:id="GymoryHyperlink1502"/>
+    <x:hyperlink ref="H622" r:id="GymoryHyperlink1503"/>
+    <x:hyperlink ref="I622" r:id="GymoryHyperlink1504"/>
+    <x:hyperlink ref="J622" r:id="GymoryHyperlink1505"/>
+    <x:hyperlink ref="H623" r:id="GymoryHyperlink1506"/>
+    <x:hyperlink ref="I623" r:id="GymoryHyperlink1507"/>
+    <x:hyperlink ref="J623" r:id="GymoryHyperlink1508"/>
+    <x:hyperlink ref="H624" r:id="GymoryHyperlink1509"/>
+    <x:hyperlink ref="I624" r:id="GymoryHyperlink1510"/>
+    <x:hyperlink ref="J624" r:id="GymoryHyperlink1511"/>
+    <x:hyperlink ref="H625" r:id="GymoryHyperlink1512"/>
+    <x:hyperlink ref="I625" r:id="GymoryHyperlink1513"/>
+    <x:hyperlink ref="J625" r:id="GymoryHyperlink1514"/>
+    <x:hyperlink ref="H626" r:id="GymoryHyperlink1515"/>
+    <x:hyperlink ref="I626" r:id="GymoryHyperlink1516"/>
+    <x:hyperlink ref="J626" r:id="GymoryHyperlink1517"/>
+    <x:hyperlink ref="H627" r:id="GymoryHyperlink1518"/>
+    <x:hyperlink ref="I627" r:id="GymoryHyperlink1519"/>
+    <x:hyperlink ref="J627" r:id="GymoryHyperlink1520"/>
+    <x:hyperlink ref="H628" r:id="GymoryHyperlink1521"/>
+    <x:hyperlink ref="I628" r:id="GymoryHyperlink1522"/>
+    <x:hyperlink ref="J628" r:id="GymoryHyperlink1523"/>
+    <x:hyperlink ref="H629" r:id="GymoryHyperlink1524"/>
+    <x:hyperlink ref="I629" r:id="GymoryHyperlink1525"/>
+    <x:hyperlink ref="J629" r:id="GymoryHyperlink1526"/>
+    <x:hyperlink ref="H630" r:id="GymoryHyperlink1527"/>
+    <x:hyperlink ref="I630" r:id="GymoryHyperlink1528"/>
+    <x:hyperlink ref="J630" r:id="GymoryHyperlink1529"/>
+    <x:hyperlink ref="H631" r:id="GymoryHyperlink1530"/>
+    <x:hyperlink ref="I631" r:id="GymoryHyperlink1531"/>
+    <x:hyperlink ref="J631" r:id="GymoryHyperlink1532"/>
+    <x:hyperlink ref="H632" r:id="GymoryHyperlink1533"/>
+    <x:hyperlink ref="I632" r:id="GymoryHyperlink1534"/>
+    <x:hyperlink ref="J632" r:id="GymoryHyperlink1535"/>
+    <x:hyperlink ref="H633" r:id="GymoryHyperlink1536"/>
+    <x:hyperlink ref="I633" r:id="GymoryHyperlink1537"/>
+    <x:hyperlink ref="J633" r:id="GymoryHyperlink1538"/>
+    <x:hyperlink ref="H634" r:id="GymoryHyperlink1539"/>
+    <x:hyperlink ref="I634" r:id="GymoryHyperlink1540"/>
+    <x:hyperlink ref="J634" r:id="GymoryHyperlink1541"/>
+    <x:hyperlink ref="H635" r:id="GymoryHyperlink1542"/>
+    <x:hyperlink ref="I635" r:id="GymoryHyperlink1543"/>
+    <x:hyperlink ref="J635" r:id="GymoryHyperlink1544"/>
+    <x:hyperlink ref="H636" r:id="GymoryHyperlink1545"/>
+    <x:hyperlink ref="I636" r:id="GymoryHyperlink1546"/>
+    <x:hyperlink ref="J636" r:id="GymoryHyperlink1547"/>
+    <x:hyperlink ref="H637" r:id="GymoryHyperlink1548"/>
+    <x:hyperlink ref="I637" r:id="GymoryHyperlink1549"/>
+    <x:hyperlink ref="J637" r:id="GymoryHyperlink1550"/>
+    <x:hyperlink ref="H638" r:id="GymoryHyperlink1551"/>
+    <x:hyperlink ref="I638" r:id="GymoryHyperlink1552"/>
+    <x:hyperlink ref="J638" r:id="GymoryHyperlink1553"/>
+    <x:hyperlink ref="H639" r:id="GymoryHyperlink1554"/>
+    <x:hyperlink ref="I639" r:id="GymoryHyperlink1555"/>
+    <x:hyperlink ref="J639" r:id="GymoryHyperlink1556"/>
+    <x:hyperlink ref="H640" r:id="GymoryHyperlink1557"/>
+    <x:hyperlink ref="I640" r:id="GymoryHyperlink1558"/>
+    <x:hyperlink ref="J640" r:id="GymoryHyperlink1559"/>
+    <x:hyperlink ref="H641" r:id="GymoryHyperlink1560"/>
+    <x:hyperlink ref="I641" r:id="GymoryHyperlink1561"/>
+    <x:hyperlink ref="J641" r:id="GymoryHyperlink1562"/>
+    <x:hyperlink ref="H642" r:id="GymoryHyperlink1563"/>
+    <x:hyperlink ref="I642" r:id="GymoryHyperlink1564"/>
+    <x:hyperlink ref="J642" r:id="GymoryHyperlink1565"/>
+    <x:hyperlink ref="H643" r:id="GymoryHyperlink1566"/>
+    <x:hyperlink ref="I643" r:id="GymoryHyperlink1567"/>
+    <x:hyperlink ref="J643" r:id="GymoryHyperlink1568"/>
+    <x:hyperlink ref="H644" r:id="GymoryHyperlink1569"/>
+    <x:hyperlink ref="I644" r:id="GymoryHyperlink1570"/>
+    <x:hyperlink ref="J644" r:id="GymoryHyperlink1571"/>
+    <x:hyperlink ref="H645" r:id="GymoryHyperlink1572"/>
+    <x:hyperlink ref="I645" r:id="GymoryHyperlink1573"/>
+    <x:hyperlink ref="J645" r:id="GymoryHyperlink1574"/>
+    <x:hyperlink ref="J646" r:id="GymoryHyperlink1575"/>
+    <x:hyperlink ref="H647" r:id="GymoryHyperlink1576"/>
+    <x:hyperlink ref="I647" r:id="GymoryHyperlink1577"/>
+    <x:hyperlink ref="J647" r:id="GymoryHyperlink1578"/>
+    <x:hyperlink ref="J648" r:id="GymoryHyperlink1579"/>
+    <x:hyperlink ref="J649" r:id="GymoryHyperlink1580"/>
+    <x:hyperlink ref="J650" r:id="GymoryHyperlink1581"/>
+    <x:hyperlink ref="H651" r:id="GymoryHyperlink1582"/>
+    <x:hyperlink ref="I651" r:id="GymoryHyperlink1583"/>
+    <x:hyperlink ref="J651" r:id="GymoryHyperlink1584"/>
+    <x:hyperlink ref="H652" r:id="GymoryHyperlink1585"/>
+    <x:hyperlink ref="I652" r:id="GymoryHyperlink1586"/>
+    <x:hyperlink ref="J652" r:id="GymoryHyperlink1587"/>
+    <x:hyperlink ref="H653" r:id="GymoryHyperlink1588"/>
+    <x:hyperlink ref="I653" r:id="GymoryHyperlink1589"/>
+    <x:hyperlink ref="J653" r:id="GymoryHyperlink1590"/>
+    <x:hyperlink ref="H654" r:id="GymoryHyperlink1591"/>
+    <x:hyperlink ref="I654" r:id="GymoryHyperlink1592"/>
+    <x:hyperlink ref="J654" r:id="GymoryHyperlink1593"/>
+    <x:hyperlink ref="H655" r:id="GymoryHyperlink1594"/>
+    <x:hyperlink ref="I655" r:id="GymoryHyperlink1595"/>
+    <x:hyperlink ref="J655" r:id="GymoryHyperlink1596"/>
+    <x:hyperlink ref="H656" r:id="GymoryHyperlink1597"/>
+    <x:hyperlink ref="I656" r:id="GymoryHyperlink1598"/>
+    <x:hyperlink ref="J656" r:id="GymoryHyperlink1599"/>
+    <x:hyperlink ref="H657" r:id="GymoryHyperlink1600"/>
+    <x:hyperlink ref="I657" r:id="GymoryHyperlink1601"/>
+    <x:hyperlink ref="J657" r:id="GymoryHyperlink1602"/>
+    <x:hyperlink ref="H658" r:id="GymoryHyperlink1603"/>
+    <x:hyperlink ref="I658" r:id="GymoryHyperlink1604"/>
+    <x:hyperlink ref="J658" r:id="GymoryHyperlink1605"/>
+    <x:hyperlink ref="J659" r:id="GymoryHyperlink1606"/>
+    <x:hyperlink ref="H660" r:id="GymoryHyperlink1607"/>
+    <x:hyperlink ref="I660" r:id="GymoryHyperlink1608"/>
+    <x:hyperlink ref="J660" r:id="GymoryHyperlink1609"/>
+    <x:hyperlink ref="H661" r:id="GymoryHyperlink1610"/>
+    <x:hyperlink ref="I661" r:id="GymoryHyperlink1611"/>
+    <x:hyperlink ref="J661" r:id="GymoryHyperlink1612"/>
+    <x:hyperlink ref="H662" r:id="GymoryHyperlink1613"/>
+    <x:hyperlink ref="I662" r:id="GymoryHyperlink1614"/>
+    <x:hyperlink ref="J662" r:id="GymoryHyperlink1615"/>
+    <x:hyperlink ref="H663" r:id="GymoryHyperlink1616"/>
+    <x:hyperlink ref="I663" r:id="GymoryHyperlink1617"/>
+    <x:hyperlink ref="J663" r:id="GymoryHyperlink1618"/>
+    <x:hyperlink ref="H664" r:id="GymoryHyperlink1619"/>
+    <x:hyperlink ref="I664" r:id="GymoryHyperlink1620"/>
+    <x:hyperlink ref="J664" r:id="GymoryHyperlink1621"/>
+    <x:hyperlink ref="H665" r:id="GymoryHyperlink1622"/>
+    <x:hyperlink ref="I665" r:id="GymoryHyperlink1623"/>
+    <x:hyperlink ref="J665" r:id="GymoryHyperlink1624"/>
+    <x:hyperlink ref="J666" r:id="GymoryHyperlink1625"/>
+    <x:hyperlink ref="K666" r:id="GymoryHyperlink1626"/>
+    <x:hyperlink ref="J667" r:id="GymoryHyperlink1627"/>
+    <x:hyperlink ref="J668" r:id="GymoryHyperlink1628"/>
+    <x:hyperlink ref="K668" r:id="GymoryHyperlink1629"/>
+    <x:hyperlink ref="J669" r:id="GymoryHyperlink1630"/>
+    <x:hyperlink ref="K669" r:id="GymoryHyperlink1631"/>
+    <x:hyperlink ref="J670" r:id="GymoryHyperlink1632"/>
+    <x:hyperlink ref="K670" r:id="GymoryHyperlink1633"/>
+    <x:hyperlink ref="H671" r:id="GymoryHyperlink1634"/>
+    <x:hyperlink ref="I671" r:id="GymoryHyperlink1635"/>
+    <x:hyperlink ref="J671" r:id="GymoryHyperlink1636"/>
+    <x:hyperlink ref="J672" r:id="GymoryHyperlink1637"/>
+    <x:hyperlink ref="K672" r:id="GymoryHyperlink1638"/>
+    <x:hyperlink ref="H673" r:id="GymoryHyperlink1639"/>
+    <x:hyperlink ref="I673" r:id="GymoryHyperlink1640"/>
+    <x:hyperlink ref="J673" r:id="GymoryHyperlink1641"/>
+    <x:hyperlink ref="H674" r:id="GymoryHyperlink1642"/>
+    <x:hyperlink ref="I674" r:id="GymoryHyperlink1643"/>
+    <x:hyperlink ref="J674" r:id="GymoryHyperlink1644"/>
+    <x:hyperlink ref="H675" r:id="GymoryHyperlink1645"/>
+    <x:hyperlink ref="I675" r:id="GymoryHyperlink1646"/>
+    <x:hyperlink ref="J675" r:id="GymoryHyperlink1647"/>
+    <x:hyperlink ref="H676" r:id="GymoryHyperlink1648"/>
+    <x:hyperlink ref="I676" r:id="GymoryHyperlink1649"/>
+    <x:hyperlink ref="J676" r:id="GymoryHyperlink1650"/>
+    <x:hyperlink ref="H677" r:id="GymoryHyperlink1651"/>
+    <x:hyperlink ref="I677" r:id="GymoryHyperlink1652"/>
+    <x:hyperlink ref="J677" r:id="GymoryHyperlink1653"/>
+    <x:hyperlink ref="H678" r:id="GymoryHyperlink1654"/>
+    <x:hyperlink ref="I678" r:id="GymoryHyperlink1655"/>
+    <x:hyperlink ref="J678" r:id="GymoryHyperlink1656"/>
+    <x:hyperlink ref="H679" r:id="GymoryHyperlink1657"/>
+    <x:hyperlink ref="I679" r:id="GymoryHyperlink1658"/>
+    <x:hyperlink ref="J679" r:id="GymoryHyperlink1659"/>
+    <x:hyperlink ref="H680" r:id="GymoryHyperlink1660"/>
+    <x:hyperlink ref="I680" r:id="GymoryHyperlink1661"/>
+    <x:hyperlink ref="J680" r:id="GymoryHyperlink1662"/>
+    <x:hyperlink ref="J681" r:id="GymoryHyperlink1663"/>
+    <x:hyperlink ref="K681" r:id="GymoryHyperlink1664"/>
+    <x:hyperlink ref="J682" r:id="GymoryHyperlink1665"/>
+    <x:hyperlink ref="K682" r:id="GymoryHyperlink1666"/>
+    <x:hyperlink ref="J683" r:id="GymoryHyperlink1667"/>
+    <x:hyperlink ref="J684" r:id="GymoryHyperlink1668"/>
+    <x:hyperlink ref="J685" r:id="GymoryHyperlink1669"/>
+    <x:hyperlink ref="K685" r:id="GymoryHyperlink1670"/>
+    <x:hyperlink ref="H686" r:id="GymoryHyperlink1671"/>
+    <x:hyperlink ref="I686" r:id="GymoryHyperlink1672"/>
+    <x:hyperlink ref="J686" r:id="GymoryHyperlink1673"/>
+    <x:hyperlink ref="J687" r:id="GymoryHyperlink1674"/>
+    <x:hyperlink ref="H688" r:id="GymoryHyperlink1675"/>
+    <x:hyperlink ref="I688" r:id="GymoryHyperlink1676"/>
+    <x:hyperlink ref="J688" r:id="GymoryHyperlink1677"/>
+    <x:hyperlink ref="J689" r:id="GymoryHyperlink1678"/>
+    <x:hyperlink ref="H690" r:id="GymoryHyperlink1679"/>
+    <x:hyperlink ref="I690" r:id="GymoryHyperlink1680"/>
+    <x:hyperlink ref="J690" r:id="GymoryHyperlink1681"/>
+    <x:hyperlink ref="J691" r:id="GymoryHyperlink1682"/>
+    <x:hyperlink ref="H692" r:id="GymoryHyperlink1683"/>
+    <x:hyperlink ref="I692" r:id="GymoryHyperlink1684"/>
+    <x:hyperlink ref="J692" r:id="GymoryHyperlink1685"/>
+    <x:hyperlink ref="J693" r:id="GymoryHyperlink1686"/>
+    <x:hyperlink ref="K693" r:id="GymoryHyperlink1687"/>
+    <x:hyperlink ref="J694" r:id="GymoryHyperlink1688"/>
+    <x:hyperlink ref="K694" r:id="GymoryHyperlink1689"/>
+    <x:hyperlink ref="J695" r:id="GymoryHyperlink1690"/>
+    <x:hyperlink ref="J696" r:id="GymoryHyperlink1691"/>
+    <x:hyperlink ref="K696" r:id="GymoryHyperlink1692"/>
+    <x:hyperlink ref="J697" r:id="GymoryHyperlink1693"/>
+    <x:hyperlink ref="K697" r:id="GymoryHyperlink1694"/>
+    <x:hyperlink ref="J698" r:id="GymoryHyperlink1695"/>
+    <x:hyperlink ref="K698" r:id="GymoryHyperlink1696"/>
+    <x:hyperlink ref="J699" r:id="GymoryHyperlink1697"/>
+    <x:hyperlink ref="K699" r:id="GymoryHyperlink1698"/>
+    <x:hyperlink ref="J700" r:id="GymoryHyperlink1699"/>
+    <x:hyperlink ref="K700" r:id="GymoryHyperlink1700"/>
+    <x:hyperlink ref="J701" r:id="GymoryHyperlink1701"/>
+    <x:hyperlink ref="K701" r:id="GymoryHyperlink1702"/>
+    <x:hyperlink ref="J702" r:id="GymoryHyperlink1703"/>
+    <x:hyperlink ref="K702" r:id="GymoryHyperlink1704"/>
+    <x:hyperlink ref="J703" r:id="GymoryHyperlink1705"/>
+    <x:hyperlink ref="K703" r:id="GymoryHyperlink1706"/>
+    <x:hyperlink ref="J704" r:id="GymoryHyperlink1707"/>
+    <x:hyperlink ref="K704" r:id="GymoryHyperlink1708"/>
+    <x:hyperlink ref="J705" r:id="GymoryHyperlink1709"/>
+    <x:hyperlink ref="K705" r:id="GymoryHyperlink1710"/>
+    <x:hyperlink ref="J706" r:id="GymoryHyperlink1711"/>
+    <x:hyperlink ref="K706" r:id="GymoryHyperlink1712"/>
+    <x:hyperlink ref="J707" r:id="GymoryHyperlink1713"/>
+    <x:hyperlink ref="J708" r:id="GymoryHyperlink1714"/>
+    <x:hyperlink ref="J709" r:id="GymoryHyperlink1715"/>
+    <x:hyperlink ref="J710" r:id="GymoryHyperlink1716"/>
+    <x:hyperlink ref="H711" r:id="GymoryHyperlink1717"/>
+    <x:hyperlink ref="I711" r:id="GymoryHyperlink1718"/>
+    <x:hyperlink ref="J711" r:id="GymoryHyperlink1719"/>
+    <x:hyperlink ref="H712" r:id="GymoryHyperlink1720"/>
+    <x:hyperlink ref="I712" r:id="GymoryHyperlink1721"/>
+    <x:hyperlink ref="J712" r:id="GymoryHyperlink1722"/>
+    <x:hyperlink ref="H713" r:id="GymoryHyperlink1723"/>
+    <x:hyperlink ref="I713" r:id="GymoryHyperlink1724"/>
+    <x:hyperlink ref="J713" r:id="GymoryHyperlink1725"/>
+    <x:hyperlink ref="H714" r:id="GymoryHyperlink1726"/>
+    <x:hyperlink ref="I714" r:id="GymoryHyperlink1727"/>
+    <x:hyperlink ref="J714" r:id="GymoryHyperlink1728"/>
+    <x:hyperlink ref="H715" r:id="GymoryHyperlink1729"/>
+    <x:hyperlink ref="I715" r:id="GymoryHyperlink1730"/>
+    <x:hyperlink ref="J715" r:id="GymoryHyperlink1731"/>
+    <x:hyperlink ref="J716" r:id="GymoryHyperlink1732"/>
+    <x:hyperlink ref="K716" r:id="GymoryHyperlink1733"/>
+    <x:hyperlink ref="H717" r:id="GymoryHyperlink1734"/>
+    <x:hyperlink ref="I717" r:id="GymoryHyperlink1735"/>
+    <x:hyperlink ref="J717" r:id="GymoryHyperlink1736"/>
+    <x:hyperlink ref="H718" r:id="GymoryHyperlink1737"/>
+    <x:hyperlink ref="I718" r:id="GymoryHyperlink1738"/>
+    <x:hyperlink ref="J718" r:id="GymoryHyperlink1739"/>
+    <x:hyperlink ref="H719" r:id="GymoryHyperlink1740"/>
+    <x:hyperlink ref="I719" r:id="GymoryHyperlink1741"/>
+    <x:hyperlink ref="J719" r:id="GymoryHyperlink1742"/>
+    <x:hyperlink ref="H720" r:id="GymoryHyperlink1743"/>
+    <x:hyperlink ref="I720" r:id="GymoryHyperlink1744"/>
+    <x:hyperlink ref="J720" r:id="GymoryHyperlink1745"/>
+    <x:hyperlink ref="H721" r:id="GymoryHyperlink1746"/>
+    <x:hyperlink ref="I721" r:id="GymoryHyperlink1747"/>
+    <x:hyperlink ref="J721" r:id="GymoryHyperlink1748"/>
+    <x:hyperlink ref="H722" r:id="GymoryHyperlink1749"/>
+    <x:hyperlink ref="I722" r:id="GymoryHyperlink1750"/>
+    <x:hyperlink ref="J722" r:id="GymoryHyperlink1751"/>
+    <x:hyperlink ref="H723" r:id="GymoryHyperlink1752"/>
+    <x:hyperlink ref="I723" r:id="GymoryHyperlink1753"/>
+    <x:hyperlink ref="J723" r:id="GymoryHyperlink1754"/>
+    <x:hyperlink ref="H724" r:id="GymoryHyperlink1755"/>
+    <x:hyperlink ref="I724" r:id="GymoryHyperlink1756"/>
+    <x:hyperlink ref="J724" r:id="GymoryHyperlink1757"/>
+    <x:hyperlink ref="H725" r:id="GymoryHyperlink1758"/>
+    <x:hyperlink ref="I725" r:id="GymoryHyperlink1759"/>
+    <x:hyperlink ref="J725" r:id="GymoryHyperlink1760"/>
+    <x:hyperlink ref="H726" r:id="GymoryHyperlink1761"/>
+    <x:hyperlink ref="I726" r:id="GymoryHyperlink1762"/>
+    <x:hyperlink ref="J726" r:id="GymoryHyperlink1763"/>
+    <x:hyperlink ref="H727" r:id="GymoryHyperlink1764"/>
+    <x:hyperlink ref="I727" r:id="GymoryHyperlink1765"/>
+    <x:hyperlink ref="J727" r:id="GymoryHyperlink1766"/>
+    <x:hyperlink ref="H728" r:id="GymoryHyperlink1767"/>
+    <x:hyperlink ref="I728" r:id="GymoryHyperlink1768"/>
+    <x:hyperlink ref="J728" r:id="GymoryHyperlink1769"/>
+    <x:hyperlink ref="J729" r:id="GymoryHyperlink1770"/>
+    <x:hyperlink ref="K729" r:id="GymoryHyperlink1771"/>
+    <x:hyperlink ref="J730" r:id="GymoryHyperlink1772"/>
+    <x:hyperlink ref="K730" r:id="GymoryHyperlink1773"/>
+    <x:hyperlink ref="J731" r:id="GymoryHyperlink1774"/>
+    <x:hyperlink ref="K731" r:id="GymoryHyperlink1775"/>
+    <x:hyperlink ref="H732" r:id="GymoryHyperlink1776"/>
+    <x:hyperlink ref="I732" r:id="GymoryHyperlink1777"/>
+    <x:hyperlink ref="J732" r:id="GymoryHyperlink1778"/>
+    <x:hyperlink ref="H733" r:id="GymoryHyperlink1779"/>
+    <x:hyperlink ref="I733" r:id="GymoryHyperlink1780"/>
+    <x:hyperlink ref="J733" r:id="GymoryHyperlink1781"/>
+    <x:hyperlink ref="J734" r:id="GymoryHyperlink1782"/>
+    <x:hyperlink ref="K734" r:id="GymoryHyperlink1783"/>
+    <x:hyperlink ref="J735" r:id="GymoryHyperlink1784"/>
+    <x:hyperlink ref="K735" r:id="GymoryHyperlink1785"/>
+    <x:hyperlink ref="J736" r:id="GymoryHyperlink1786"/>
+    <x:hyperlink ref="H737" r:id="GymoryHyperlink1787"/>
+    <x:hyperlink ref="I737" r:id="GymoryHyperlink1788"/>
+    <x:hyperlink ref="J737" r:id="GymoryHyperlink1789"/>
+    <x:hyperlink ref="H738" r:id="GymoryHyperlink1790"/>
+    <x:hyperlink ref="I738" r:id="GymoryHyperlink1791"/>
+    <x:hyperlink ref="J738" r:id="GymoryHyperlink1792"/>
+    <x:hyperlink ref="H739" r:id="GymoryHyperlink1793"/>
+    <x:hyperlink ref="I739" r:id="GymoryHyperlink1794"/>
+    <x:hyperlink ref="J739" r:id="GymoryHyperlink1795"/>
+    <x:hyperlink ref="H740" r:id="GymoryHyperlink1796"/>
+    <x:hyperlink ref="I740" r:id="GymoryHyperlink1797"/>
+    <x:hyperlink ref="J740" r:id="GymoryHyperlink1798"/>
+    <x:hyperlink ref="H741" r:id="GymoryHyperlink1799"/>
+    <x:hyperlink ref="I741" r:id="GymoryHyperlink1800"/>
+    <x:hyperlink ref="J741" r:id="GymoryHyperlink1801"/>
+    <x:hyperlink ref="H742" r:id="GymoryHyperlink1802"/>
+    <x:hyperlink ref="I742" r:id="GymoryHyperlink1803"/>
+    <x:hyperlink ref="J742" r:id="GymoryHyperlink1804"/>
+    <x:hyperlink ref="H743" r:id="GymoryHyperlink1805"/>
+    <x:hyperlink ref="I743" r:id="GymoryHyperlink1806"/>
+    <x:hyperlink ref="J743" r:id="GymoryHyperlink1807"/>
+    <x:hyperlink ref="H744" r:id="GymoryHyperlink1808"/>
+    <x:hyperlink ref="I744" r:id="GymoryHyperlink1809"/>
+    <x:hyperlink ref="J744" r:id="GymoryHyperlink1810"/>
+    <x:hyperlink ref="H745" r:id="GymoryHyperlink1811"/>
+    <x:hyperlink ref="I745" r:id="GymoryHyperlink1812"/>
+    <x:hyperlink ref="J745" r:id="GymoryHyperlink1813"/>
+    <x:hyperlink ref="H746" r:id="GymoryHyperlink1814"/>
+    <x:hyperlink ref="I746" r:id="GymoryHyperlink1815"/>
+    <x:hyperlink ref="J746" r:id="GymoryHyperlink1816"/>
+    <x:hyperlink ref="H747" r:id="GymoryHyperlink1817"/>
+    <x:hyperlink ref="I747" r:id="GymoryHyperlink1818"/>
+    <x:hyperlink ref="J747" r:id="GymoryHyperlink1819"/>
+    <x:hyperlink ref="H748" r:id="GymoryHyperlink1820"/>
+    <x:hyperlink ref="I748" r:id="GymoryHyperlink1821"/>
+    <x:hyperlink ref="J748" r:id="GymoryHyperlink1822"/>
+    <x:hyperlink ref="H749" r:id="GymoryHyperlink1823"/>
+    <x:hyperlink ref="I749" r:id="GymoryHyperlink1824"/>
+    <x:hyperlink ref="J749" r:id="GymoryHyperlink1825"/>
+    <x:hyperlink ref="H750" r:id="GymoryHyperlink1826"/>
+    <x:hyperlink ref="I750" r:id="GymoryHyperlink1827"/>
+    <x:hyperlink ref="J750" r:id="GymoryHyperlink1828"/>
+    <x:hyperlink ref="H751" r:id="GymoryHyperlink1829"/>
+    <x:hyperlink ref="I751" r:id="GymoryHyperlink1830"/>
+    <x:hyperlink ref="J751" r:id="GymoryHyperlink1831"/>
+    <x:hyperlink ref="H752" r:id="GymoryHyperlink1832"/>
+    <x:hyperlink ref="I752" r:id="GymoryHyperlink1833"/>
+    <x:hyperlink ref="J752" r:id="GymoryHyperlink1834"/>
+    <x:hyperlink ref="H753" r:id="GymoryHyperlink1835"/>
+    <x:hyperlink ref="I753" r:id="GymoryHyperlink1836"/>
+    <x:hyperlink ref="J753" r:id="GymoryHyperlink1837"/>
+    <x:hyperlink ref="H754" r:id="GymoryHyperlink1838"/>
+    <x:hyperlink ref="I754" r:id="GymoryHyperlink1839"/>
+    <x:hyperlink ref="J754" r:id="GymoryHyperlink1840"/>
+    <x:hyperlink ref="H755" r:id="GymoryHyperlink1841"/>
+    <x:hyperlink ref="I755" r:id="GymoryHyperlink1842"/>
+    <x:hyperlink ref="J755" r:id="GymoryHyperlink1843"/>
+    <x:hyperlink ref="H756" r:id="GymoryHyperlink1844"/>
+    <x:hyperlink ref="I756" r:id="GymoryHyperlink1845"/>
+    <x:hyperlink ref="J756" r:id="GymoryHyperlink1846"/>
+    <x:hyperlink ref="J757" r:id="GymoryHyperlink1847"/>
+    <x:hyperlink ref="J758" r:id="GymoryHyperlink1848"/>
+    <x:hyperlink ref="J759" r:id="GymoryHyperlink1849"/>
+    <x:hyperlink ref="J760" r:id="GymoryHyperlink1850"/>
+    <x:hyperlink ref="J761" r:id="GymoryHyperlink1851"/>
+    <x:hyperlink ref="J762" r:id="GymoryHyperlink1852"/>
+    <x:hyperlink ref="K762" r:id="GymoryHyperlink1853"/>
+    <x:hyperlink ref="J763" r:id="GymoryHyperlink1854"/>
+    <x:hyperlink ref="J764" r:id="GymoryHyperlink1855"/>
+    <x:hyperlink ref="K764" r:id="GymoryHyperlink1856"/>
+    <x:hyperlink ref="J765" r:id="GymoryHyperlink1857"/>
+    <x:hyperlink ref="J766" r:id="GymoryHyperlink1858"/>
+    <x:hyperlink ref="K766" r:id="GymoryHyperlink1859"/>
+    <x:hyperlink ref="H767" r:id="GymoryHyperlink1860"/>
+    <x:hyperlink ref="I767" r:id="GymoryHyperlink1861"/>
+    <x:hyperlink ref="J767" r:id="GymoryHyperlink1862"/>
+    <x:hyperlink ref="J768" r:id="GymoryHyperlink1863"/>
+    <x:hyperlink ref="J769" r:id="GymoryHyperlink1864"/>
+    <x:hyperlink ref="J770" r:id="GymoryHyperlink1865"/>
+    <x:hyperlink ref="J771" r:id="GymoryHyperlink1866"/>
+    <x:hyperlink ref="J772" r:id="GymoryHyperlink1867"/>
+    <x:hyperlink ref="J773" r:id="GymoryHyperlink1868"/>
+    <x:hyperlink ref="J774" r:id="GymoryHyperlink1869"/>
+    <x:hyperlink ref="J775" r:id="GymoryHyperlink1870"/>
+    <x:hyperlink ref="K775" r:id="GymoryHyperlink1871"/>
+    <x:hyperlink ref="J776" r:id="GymoryHyperlink1872"/>
+    <x:hyperlink ref="J777" r:id="GymoryHyperlink1873"/>
+    <x:hyperlink ref="J778" r:id="GymoryHyperlink1874"/>
+    <x:hyperlink ref="J779" r:id="GymoryHyperlink1875"/>
+    <x:hyperlink ref="J780" r:id="GymoryHyperlink1876"/>
+    <x:hyperlink ref="J781" r:id="GymoryHyperlink1877"/>
+    <x:hyperlink ref="J782" r:id="GymoryHyperlink1878"/>
+    <x:hyperlink ref="J783" r:id="GymoryHyperlink1879"/>
+    <x:hyperlink ref="J784" r:id="GymoryHyperlink1880"/>
+    <x:hyperlink ref="J785" r:id="GymoryHyperlink1881"/>
+    <x:hyperlink ref="J786" r:id="GymoryHyperlink1882"/>
+    <x:hyperlink ref="J787" r:id="GymoryHyperlink1883"/>
+    <x:hyperlink ref="J788" r:id="GymoryHyperlink1884"/>
+    <x:hyperlink ref="J789" r:id="GymoryHyperlink1885"/>
+    <x:hyperlink ref="J790" r:id="GymoryHyperlink1886"/>
+    <x:hyperlink ref="J791" r:id="GymoryHyperlink1887"/>
+    <x:hyperlink ref="J792" r:id="GymoryHyperlink1888"/>
+    <x:hyperlink ref="J793" r:id="GymoryHyperlink1889"/>
+    <x:hyperlink ref="J794" r:id="GymoryHyperlink1890"/>
+    <x:hyperlink ref="K794" r:id="GymoryHyperlink1891"/>
+    <x:hyperlink ref="J795" r:id="GymoryHyperlink1892"/>
+    <x:hyperlink ref="J796" r:id="GymoryHyperlink1893"/>
+    <x:hyperlink ref="J797" r:id="GymoryHyperlink1894"/>
+    <x:hyperlink ref="J798" r:id="GymoryHyperlink1895"/>
+    <x:hyperlink ref="J799" r:id="GymoryHyperlink1896"/>
+    <x:hyperlink ref="J800" r:id="GymoryHyperlink1897"/>
+    <x:hyperlink ref="J801" r:id="GymoryHyperlink1898"/>
+    <x:hyperlink ref="J802" r:id="GymoryHyperlink1899"/>
+    <x:hyperlink ref="J803" r:id="GymoryHyperlink1900"/>
+    <x:hyperlink ref="J804" r:id="GymoryHyperlink1901"/>
+    <x:hyperlink ref="J805" r:id="GymoryHyperlink1902"/>
+    <x:hyperlink ref="J806" r:id="GymoryHyperlink1903"/>
+    <x:hyperlink ref="J807" r:id="GymoryHyperlink1904"/>
+    <x:hyperlink ref="K807" r:id="GymoryHyperlink1905"/>
+    <x:hyperlink ref="J808" r:id="GymoryHyperlink1906"/>
+    <x:hyperlink ref="J809" r:id="GymoryHyperlink1907"/>
+    <x:hyperlink ref="J810" r:id="GymoryHyperlink1908"/>
+    <x:hyperlink ref="J811" r:id="GymoryHyperlink1909"/>
+    <x:hyperlink ref="J812" r:id="GymoryHyperlink1910"/>
+    <x:hyperlink ref="J813" r:id="GymoryHyperlink1911"/>
+    <x:hyperlink ref="J814" r:id="GymoryHyperlink1912"/>
+    <x:hyperlink ref="J815" r:id="GymoryHyperlink1913"/>
+    <x:hyperlink ref="J816" r:id="GymoryHyperlink1914"/>
+    <x:hyperlink ref="J817" r:id="GymoryHyperlink1915"/>
+    <x:hyperlink ref="J818" r:id="GymoryHyperlink1916"/>
+    <x:hyperlink ref="J819" r:id="GymoryHyperlink1917"/>
+    <x:hyperlink ref="J820" r:id="GymoryHyperlink1918"/>
+    <x:hyperlink ref="J821" r:id="GymoryHyperlink1919"/>
+    <x:hyperlink ref="J822" r:id="GymoryHyperlink1920"/>
+    <x:hyperlink ref="J823" r:id="GymoryHyperlink1921"/>
+    <x:hyperlink ref="J824" r:id="GymoryHyperlink1922"/>
+    <x:hyperlink ref="J825" r:id="GymoryHyperlink1923"/>
+    <x:hyperlink ref="J826" r:id="GymoryHyperlink1924"/>
+    <x:hyperlink ref="J827" r:id="GymoryHyperlink1925"/>
+    <x:hyperlink ref="K827" r:id="GymoryHyperlink1926"/>
+    <x:hyperlink ref="J828" r:id="GymoryHyperlink1927"/>
+    <x:hyperlink ref="J829" r:id="GymoryHyperlink1928"/>
+    <x:hyperlink ref="J830" r:id="GymoryHyperlink1929"/>
+    <x:hyperlink ref="J831" r:id="GymoryHyperlink1930"/>
+    <x:hyperlink ref="J832" r:id="GymoryHyperlink1931"/>
+    <x:hyperlink ref="K832" r:id="GymoryHyperlink1932"/>
+    <x:hyperlink ref="J833" r:id="GymoryHyperlink1933"/>
+    <x:hyperlink ref="K833" r:id="GymoryHyperlink1934"/>
+    <x:hyperlink ref="J834" r:id="GymoryHyperlink1935"/>
+    <x:hyperlink ref="J835" r:id="GymoryHyperlink1936"/>
+    <x:hyperlink ref="K835" r:id="GymoryHyperlink1937"/>
+    <x:hyperlink ref="J836" r:id="GymoryHyperlink1938"/>
+    <x:hyperlink ref="K836" r:id="GymoryHyperlink1939"/>
+    <x:hyperlink ref="J837" r:id="GymoryHyperlink1940"/>
+    <x:hyperlink ref="K837" r:id="GymoryHyperlink1941"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69436b808df04225"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6be30acf100140f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>